<commit_message>
feat(wp3): add Korean knowledge graph notebook with merged relation reviews
</commit_message>
<xml_diff>
--- a/artifacts/stage1_wp3/evaluation/relation_correction/relation_review_corrected_seed2026.xlsx
+++ b/artifacts/stage1_wp3/evaluation/relation_correction/relation_review_corrected_seed2026.xlsx
@@ -714,10 +714,6 @@
           <t>BEFORE: According to independent testing from Artificial Analysis and Arena.ai, Kimi K3’s capabilities are competitive with both Anthropic’s Fable 5, which was released last month, and OpenAI’s GPT-5.6, which was released just a week prior. || EVIDENCE: Back in February, though, Anthropic accused three Chinese AI companies âMoonshot, DeepSeek, and Minimaxâ of violating Anthropic’s terms of service and regional access restrictions to “ illicitly ” extract the capabilities of its Claude model and use that to improve their own. || AFTER: Around the same time, OpenAI sent a memo to the House of Representatives, accusing DeepSeek of a similar tactic, claiming that it is trying to “ free-ride on the capabilities developed by OpenAI and other U.S. frontier labs. ”</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr">
         <is>
           <t>org:deepseek</t>
@@ -858,7 +854,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
           <t>A cloud-native suite of software tools, libraries, and frameworks accelerating production-grade AI development.</t>
@@ -886,10 +881,6 @@
           <t>BEFORE: Open-source AI is accelerating innovation across industries, and NVIDIA DGX Spark and DGX Station are built to help developers turn innovation into impact. || EVIDENCE: NVIDIA today unveiled at the CES trade show how the DGX Spark and DGX Station deskside AI supercomputers let developers harness the latest open and frontier AI models on a local deskside system, from 100-billion-parameter models on DGX Spark to 1-trillion-parameter models on DGX Station. || AFTER: Powered by the NVIDIA Grace Blackwell architecture, with large unified memory and petaflop-level AI performance, these systems give developers new capabilities to develop locally and easily scale to the cloud.</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
       <c r="Y3" t="inlineStr">
         <is>
           <t>hardware:dgx_spark</t>
@@ -1035,7 +1026,6 @@
           <t>head merged from platform:meta_platforms</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr">
         <is>
           <t>A year after spending over $ 14 billion to bring in Alexandr Wang and a group of his top Scale AI engineers to revamp its artificial intelligence efforts, Meta is at least back on the map in AI, though it's still far behind OpenAI, Anthropic and Google in the market.</t>
@@ -1057,10 +1047,6 @@
           <t>BEFORE: It comes ahead of the kickoff of Llamacon 2025, Meta’s first AI developer conference taking place this week at its office campus headquarters in Palo Alto, California, centered around its Llama model family and general AI developer tools and advances. || EVIDENCE: With the rise of more AI model challengers in the open source and proprietary domains — including everyone from OpenAI with ChatGPT to Google with its Gemini 2.5 model family and lesser-known (at least, to Western audiences) brands like Alibaba’s new Qwen 3 — Meta is keen to show off the power and capabilities of its own, in-house Llama 4 models. || AFTER: It is also seeking to make the case to third-party software developers that Llama 4 is a powerful and flexible open (ish) source model family they can trust to build their enterprise products atop of.</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr">
         <is>
           <t>org:meta</t>
@@ -1201,8 +1187,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr">
         <is>
           <t>A two-person startup by the name of Nari Labs has introduced Dia, a 1.6 billion parameter text-to-speech (TTS) model designed to produce naturalistic dialogue directly from text prompts — and one of its creators claims it surpasses the performance of competing proprietary offerings from the likes of ElevenLabs, Google’s hit NotebookLM AI podcast generation product.</t>
@@ -1221,11 +1205,6 @@
 Nari Labs, a two-person startup, released Dia, a 1.6 billion parameter text-to-speech model that generates naturalistic dialogue directly from text prompts. || EVIDENCE: The model supports advanced features like emotional tone, speaker tagging, and nonverbal audio cues such as laughs and coughs — capabilities that co-creator Toby Kim claims surpass competing offerings from ElevenLabs and Google’s NotebookLM. || AFTER: Side-by-side comparisons show Dia handling natural timing, nonverbal expressions, and emotional range quite effectively, with examples demonstrating how it properly interprets cues that other models simply read aloud or skip entirely.</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr">
         <is>
           <t>org:elevenlabs</t>
@@ -1289,9 +1268,6 @@
       <c r="AK5" t="n">
         <v>0.7022294402122498</v>
       </c>
-      <c r="AL5" t="inlineStr"/>
-      <c r="AM5" t="inlineStr"/>
-      <c r="AN5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1356,7 +1332,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
           <t>If the model delivers on promises of higher reasoning capability, better personalization and improved efficiency, it could cement OpenAI’s position as the go-to provider for both consumer and enterprise AI applications.</t>
@@ -1382,10 +1357,6 @@
           <t>BEFORE: Hold on. || EVIDENCE: Interestingly, the source code for both the V3 and R1 models and their V2 predecessor are all available on GitHub, which is more than you can say for the proprietary models from OpenAI, Google, Anthropic, xAI, and others. || AFTER: But what we want to know – and what is roiling the tech titans today – is precisely how DeepSeek was able to take a few thousand crippled “ Hopper ” H800 GPU accelerators from Nvidia, which have some of their performance capped, and create an MoE foundation model that can stand toe-to-toe with the best that OpenAI, Google, and Anthropic can do with their largest models as they are trained on tens of thousands of uncrimped GPU accelerators.</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr">
         <is>
           <t>org:google</t>
@@ -1526,7 +1497,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
           <t>The Conversational Agents console also provides new evaluation capabilities to benchmark agent performance and improve reliability and quality at scale.</t>
@@ -1548,11 +1518,6 @@
 Agent Trainer aims to boost business performance and customer satisfaction by delivering ROI through lower training costs, tailored training recommendations and faster agent proficiency—ultimately reducing turnover, Google said. || AFTER: Targeting the Contact Center-as-a-Service (CCaaS) market, Google Cloud has created a new stand-alone agent desktop application.</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
       <c r="Y7" t="inlineStr">
         <is>
           <t>person:antony_passemard</t>
@@ -1616,9 +1581,6 @@
       <c r="AK7" t="n">
         <v>0.5947865843772888</v>
       </c>
-      <c r="AL7" t="inlineStr"/>
-      <c r="AM7" t="inlineStr"/>
-      <c r="AN7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1683,7 +1645,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
           <t>FPT’s stack is beginning to take discernible form.</t>
@@ -1709,10 +1670,6 @@
           <t>BEFORE: More than $ 700 billion was wiped from the value of the world’s largest technology companies on Monday after the emergence of a cut-price Chinese rival to ChatGPT raised doubts over whether America can sustain its lead in artificial intelligence. || EVIDENCE: California-based Nvidia, whose share price has been turbocharged by speculation that generative AI would fuel rapid growth in demand for its computer chips, lost $ 590 billion, and its crown as the world’s most valuable public company. || AFTER: DeepSeek said it has produced a free open-source assistant that uses lower-cost chips and less data than its American rivals.</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr">
         <is>
           <t>org:nvidia</t>
@@ -1853,7 +1810,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
           <t>Edits in the browser update the code base, he added.</t>
@@ -1875,11 +1831,6 @@
 Bun’s frontend dev server is going to get “ automatic workspaces ” support in Chrome DevTools, which means developers can edit the files in the browser. || AFTER: Bun is a JavaScript runtime designed as a drop-in replacement for Node.js.</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
       <c r="Y9" t="inlineStr">
         <is>
           <t>product:chrome_devtools</t>
@@ -1943,9 +1894,6 @@
       <c r="AK9" t="n">
         <v>0.5579473376274109</v>
       </c>
-      <c r="AL9" t="inlineStr"/>
-      <c r="AM9" t="inlineStr"/>
-      <c r="AN9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2010,7 +1958,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
           <t>This isn’t unusual for native or web-based apps.</t>
@@ -2031,11 +1978,6 @@
           <t>EVIDENCE: BEIJING — DeepSeek's artificial intelligence breakthrough is stirring up China's venture capital world after three straight years of decline. || AFTER: As DeepSeek released its OpenAI rival in late January, AI drug discovery company Insilico Medicine was finalizing a $ 110 million series E financing round led by Hong Kong-based Value Partners, the startup's CEO and founder Alex Zhavoronkov told CNBC in an exclusive interview.</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
       <c r="Y10" t="inlineStr">
         <is>
           <t>org:deepseek</t>
@@ -2099,9 +2041,6 @@
       <c r="AK10" t="n">
         <v>0.5267133116722107</v>
       </c>
-      <c r="AL10" t="inlineStr"/>
-      <c r="AM10" t="inlineStr"/>
-      <c r="AN10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2166,8 +2105,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr">
         <is>
           <t>Meta is debuting its first major artificial intelligence model since the costly hiring of Scale AI's Alexandr Wang nine months ago, as the Facebook parent aims to carve out a niche in a market that's being dominated by OpenAI, Anthropic and Google.</t>
@@ -2188,10 +2125,6 @@
           <t>BEFORE: But those tools aren't officially available in China. || EVIDENCE: Beijing's firewall keeps out Google and Facebook and their AI models, and Anthropic cited national security concerns in its ban on China-owned entities from using Claude, widely considered the best AI for coding right now. || AFTER: Yet discussion of leading U.S. models is prevalent enough on Chinese social media to signal that such technologies are being used by local developers.</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr">
         <is>
           <t>org:facebook</t>
@@ -2332,7 +2265,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
           <t>I hope visitors will see this artwork as a way to bridge the ancient and the modern and understand the answers we seek from AI are the same as we asked from Pythia.</t>
@@ -2354,11 +2286,6 @@
           <t>BEFORE: He draws inspiration from nature and his surroundings, and attempts to capture elements of human life and the current world that we live in. || EVIDENCE: More about Polygreen Culture and Art Initiative (PCAI) and “ pi ” PCAI is a cultural organization founded by Athanasios Polychronopoulos, Polygreen CEO, as a means to increase environmental awareness through an annual programme of commissions, contemporary art exhibitions, artist residencies, workshops, conferences and sponsorships. || AFTER: The PCAI Art Collection focuses on commissions and acquisitions of moving image and contemporary art while providing artists with the means and resources to create an artwork inspired by urgent environmental, sociological and philosophical issues, allowing for their absolute freedom of expression and critical inquiry.</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
       <c r="Y12" t="inlineStr">
         <is>
           <t>org:pcai</t>
@@ -2422,9 +2349,6 @@
       <c r="AK12" t="n">
         <v>0.8922791481018066</v>
       </c>
-      <c r="AL12" t="inlineStr"/>
-      <c r="AM12" t="inlineStr"/>
-      <c r="AN12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2489,7 +2413,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
           <t>The initiative was pitched as a way to give developers more transparency and control, allowing them to host, fine-tune, and deploy the models independently.</t>
@@ -2517,10 +2440,6 @@
 While those other players do offer developer tools and products, the continual evolution of OpenAI’s developer platform makes it a hard proposition to beat as a “ one stop shop ” for those looking to leverage the latest AI advances in a clean, easy-to-use, fast and affordable way. || EVIDENCE: In a move certain to send the AI blogosphere and social media space aflutter, OpenAI is getting back into open source in a big way with the release of its Agents SDK, a toolkit designed to help developers manage, coordinate and optimize agent workflows — even building agents powered by other, non-OpenAI models such as those by competitors Anthropic and Google, or open-source models from DeepSeek, Qwen, Mistral and Meta’s Llama family. || AFTER: “ The Agent SDK is open-source, allowing enterprises to mix and match different models, ” said Godement.</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr"/>
-      <c r="X13" t="inlineStr"/>
       <c r="Y13" t="inlineStr">
         <is>
           <t>model:llama</t>
@@ -2661,7 +2580,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
           <t>The €115 million project will see the construction of “ Hunter, ” a small-scale system powered by AMD’s MI300A APUs, and “ Herder, ” a larger exascale machine designed to …</t>
@@ -2687,10 +2605,6 @@
           <t>BEFORE: However, this isn’t unique to AMD. || EVIDENCE: In MLPerf training, Nvidia has previously demonstrated a 1.3X improvement of performance over its initial “ Hopper ” H100 submissions thanks in part to software optimizations. || AFTER: With that said, driving these kinds of software optimizations are arguably even more important for AMD, which trails its rival in both market share and awareness.</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
       <c r="Y14" t="inlineStr">
         <is>
           <t>platform:hopper</t>
@@ -2831,7 +2745,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
           <t>A lot of teams are doubling down on enhancing models’ reasoning capabilities.</t>
@@ -2858,10 +2771,6 @@
 Determining which search strategy is best is still an active area of research, but there are a lot of great resources on HuggingFace which provide examples for how these search strategies can be implemented for your use case. || EVIDENCE: OpenAI’s o1 model announced in September 2024 was one of the first models designed to "think" before responding to users. || AFTER: Although it takes longer to get a response from o1 compared to models like GPT-4o, o1’s responses are typically better for more advanced tasks since it generates chain of thought sequences that help it break down and solve problems.</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
       <c r="Y15" t="inlineStr">
         <is>
           <t>model:o1_model</t>
@@ -3002,7 +2911,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
           <t>For example, the new DeepSeek-R1-Safe model was trained on 1000 Huawei Ascend chips.</t>
@@ -3023,11 +2931,6 @@
           <t>BEFORE: Far from being a “ powerful chip ” as some have claimed, the H20 actually has worse computational performance and energy efficiency than Nvidia’s older A100 chips, launched back in 2020. || EVIDENCE: Moreover, Huawei has been able to improve the computational performance of its Ascend chips, even after switching production from Taiwanese chip manufacturer TSMC to China’s own SMIC following U.S. export controls. || AFTER: Perhaps more importantly, Huawei has been making significant progress at the level of AI computing systems.</t>
         </is>
       </c>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr"/>
       <c r="Y16" t="inlineStr">
         <is>
           <t>hardware:ascend_chips</t>
@@ -3091,9 +2994,6 @@
       <c r="AK16" t="n">
         <v>0.6533774733543396</v>
       </c>
-      <c r="AL16" t="inlineStr"/>
-      <c r="AM16" t="inlineStr"/>
-      <c r="AN16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3185,11 +3085,6 @@
           <t>BEFORE: “ DeepSeek is definitely reshaping the AI landscape, challenging giants with open-source ambition and state-of-the-art innovations, ” says Kaoutar El Maghraoui, a Principal Research Scientist and Manager at IBM AI Hardware. || EVIDENCE: Meanwhile, ByteDance, the Chinese tech giant that owns TikTok, recently announced its own reasoning agent, UI-TARS, which it claims outperforms OpenAI’s GPT-4o, Anthropic’s Claude and Google’s Gemini on certain benchmarks. || AFTER: ByteDance’s agent can read graphical interfaces, reason and take autonomous, step-by-step action.</t>
         </is>
       </c>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr"/>
       <c r="Y17" t="inlineStr">
         <is>
           <t>model:gpt_4o_2</t>
@@ -3253,9 +3148,6 @@
       <c r="AK17" t="n">
         <v>0.7284291982650757</v>
       </c>
-      <c r="AL17" t="inlineStr"/>
-      <c r="AM17" t="inlineStr"/>
-      <c r="AN17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3350,10 +3242,6 @@
           <t>BEFORE: As evidenced by the tech giants’ recent announcements, the biggest AI players are unlikely to pull back on planned investments on DeepSeek’s account, Ashish Nadkarni, group vice president and general manager for worldwide infrastructure research at IDC, told Facilities Dive. || EVIDENCE: For companies like Meta and Microsoft, the drive to build as much AI capacity as quickly as possible is “ existential, ” with Apple the only major tech company to buck the trend so far, Nadkarni said. || AFTER: Those companies, and others like Elon Musk’s xAI, are using huge amounts of proprietary data to train differentiated foundational models useful in building emerging “ agentic AI ” tools and other future innovations, he added.</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr"/>
-      <c r="W18" t="inlineStr"/>
-      <c r="X18" t="inlineStr"/>
       <c r="Y18" t="inlineStr">
         <is>
           <t>org:apple</t>
@@ -3494,7 +3382,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
           <t>Now it’s back as a highly-capable workhorse for everyday use.</t>
@@ -3517,11 +3404,6 @@
 Performance: Claude Opus 5 leads many benchmarks at a cost per task lower than Claude Fable 5 but higher than most other models. || AFTER: The model’s widest performance margin came on a test of learning in unfamiliar environments.</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr"/>
-      <c r="W19" t="inlineStr"/>
-      <c r="X19" t="inlineStr"/>
       <c r="Y19" t="inlineStr">
         <is>
           <t>product:claude_opus_5</t>
@@ -3585,9 +3467,6 @@
       <c r="AK19" t="n">
         <v>0.8777515888214111</v>
       </c>
-      <c r="AL19" t="inlineStr"/>
-      <c r="AM19" t="inlineStr"/>
-      <c r="AN19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3652,7 +3531,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
           <t>Enterprises leveraging proprietary large language models (LLMs) face significant challenges that have accelerated the shift toward open-source alternatives.</t>
@@ -3679,10 +3557,6 @@
 As people across the world spend increasing amounts of time interacting with chatbots like ChatGPT, chatbot makers are struggling to work out the kind of tone and “ personality ” the models should adopt. || EVIDENCE: Back in April, OpenAI admitted it’d struck the wrong balance between helpful and sniveling, saying a new update had rendered GPT-4o too sycophantic. || AFTER: Having it suck up to you isn’t just irritating—it can mislead users by reinforcing their incorrect beliefs and spreading misinformation.</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr"/>
-      <c r="W20" t="inlineStr"/>
-      <c r="X20" t="inlineStr"/>
       <c r="Y20" t="inlineStr">
         <is>
           <t>model:gpt_4o_2</t>
@@ -3823,7 +3697,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
         <is>
           <t>Mellea is part of IBM Research’s broader vision they call “ generative computing, ” which treats language models not as magical black boxes but as computational elements that need proper software infrastructure.</t>
@@ -3844,11 +3717,6 @@
           <t>BEFORE: That’s where IBM’s Granite time series forecasting models fit in; they apply transformer technology to predict future values from time-based data. || EVIDENCE: “ Reasoning is not something a model is, it’s something a model does, ” David Cox, VP for AI models at IBM Research, told VentureBeat. || AFTER: While there has been no shortage of excitement and hype around reasoning models in 2025, reasoning for its own sake doesn’t necessarily provide value to enterprise users.</t>
         </is>
       </c>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr"/>
-      <c r="W21" t="inlineStr"/>
-      <c r="X21" t="inlineStr"/>
       <c r="Y21" t="inlineStr">
         <is>
           <t>person:david_cox</t>
@@ -3912,9 +3780,6 @@
       <c r="AK21" t="n">
         <v>0.508273184299469</v>
       </c>
-      <c r="AL21" t="inlineStr"/>
-      <c r="AM21" t="inlineStr"/>
-      <c r="AN21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3979,7 +3844,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
           <t>Five months later, distillation has suddenly become a hot-button topic from Silicon Valley to Washington, D.C., as techies and lawmakers debate whether the practice is turning into a national security threat and enabling China to catch the U.S. in the high-stakes AI race.</t>
@@ -4006,10 +3870,6 @@
 The Kimi research model even got a mention last week during Elon Musk's xAI release of Grok 4 — which scored 25.4 on its own on the "Humanity's Last Exam" benchmark, but attained a 44.4 score when allowed to use a variety of AI tools and web search.</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr"/>
-      <c r="W22" t="inlineStr"/>
-      <c r="X22" t="inlineStr"/>
       <c r="Y22" t="inlineStr">
         <is>
           <t>model:kimi</t>
@@ -4150,7 +4010,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
         <is>
           <t>DeepSeek engineers, for example, said they needed only 2,000 GPUs (graphic processing units), or chips, to train their DeepSeek-V3 model, according to a research paper they published with the model’s release.</t>
@@ -4171,11 +4030,6 @@
           <t>BEFORE: In addition, it will be “ very interesting to see the use cases they uncover for the models, ” he says. || EVIDENCE: And as IBM’s Varshney sees it, geopolitical differences may also matter less than one might assume in this global AI race. || AFTER: “ Once a model is open-sourced, where it comes from stops mattering in many respects, ” he says.</t>
         </is>
       </c>
-      <c r="T23" t="inlineStr"/>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr"/>
-      <c r="W23" t="inlineStr"/>
-      <c r="X23" t="inlineStr"/>
       <c r="Y23" t="inlineStr">
         <is>
           <t>person:kush_varshney</t>
@@ -4239,9 +4093,6 @@
       <c r="AK23" t="n">
         <v>0.5945650339126587</v>
       </c>
-      <c r="AL23" t="inlineStr"/>
-      <c r="AM23" t="inlineStr"/>
-      <c r="AN23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4306,7 +4157,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
           <t>Amazon says all of its models are faster and “ at least 75 percent less expensive ” than the best performing models in their respective intelligence classes in Amazon Bedrock (which does not host Google’s Gemini or OpenAI’s GPT models, but does host models made by AI21, Anthropic, Cohere, Meta, Mistral AI and Stability AI).</t>
@@ -4327,11 +4177,6 @@
           <t>BEFORE: Nova Premier was announced as still in training, targeted for early 2025 release. || EVIDENCE: Yes — Amazon Nova Micro, Lite and Pro are all available on Amazon Bedrock, along with Amazon Nova Canvas and Reels. || AFTER: But Amazon Nova Premier will not be available until 2025.</t>
         </is>
       </c>
-      <c r="T24" t="inlineStr"/>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr"/>
-      <c r="W24" t="inlineStr"/>
-      <c r="X24" t="inlineStr"/>
       <c r="Y24" t="inlineStr">
         <is>
           <t>product:reels</t>
@@ -4395,9 +4240,6 @@
       <c r="AK24" t="n">
         <v>0.7444586157798767</v>
       </c>
-      <c r="AL24" t="inlineStr"/>
-      <c r="AM24" t="inlineStr"/>
-      <c r="AN24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4462,7 +4304,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
           <t>”
@@ -4484,11 +4325,6 @@
           <t>BEFORE: Before Monday’s GTC keynote with NVIDIA founder and CEO Jensen Huang, catch NVIDIA GTC Live — a preshow featuring analysts, founders and industry leaders shaping the next phase of AI — starting at 8 a.m. PT. || EVIDENCE: Hosts Sarah Guo, founder of AI-native investing firm Conviction; Gavin Baker, managing partner and chief investment officer of Atreides Management; and Alfred Lin, partner at Sequoia Capital, will talk with guests about the shift from general-purpose to accelerated computing and the five-layer foundation behind one of the largest infrastructure buildouts in history. || AFTER: Correspondent Tiffany Janzen, founder of TiffinTech, will chat with guests in the crowd — including a few notable tech leaders — to get live reactions.</t>
         </is>
       </c>
-      <c r="T25" t="inlineStr"/>
-      <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr"/>
-      <c r="W25" t="inlineStr"/>
-      <c r="X25" t="inlineStr"/>
       <c r="Y25" t="inlineStr">
         <is>
           <t>org:conviction</t>
@@ -4552,9 +4388,6 @@
       <c r="AK25" t="n">
         <v>0.6532728672027588</v>
       </c>
-      <c r="AL25" t="inlineStr"/>
-      <c r="AM25" t="inlineStr"/>
-      <c r="AN25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4619,7 +4452,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
         <is>
           <t>Here are some of the most prominent hires to join Meta Superintelligence Labs:
@@ -4641,11 +4473,6 @@
           <t>BEFORE: Scale AI has made a business out of making Llama and Claude models from Anthropic consumable by and supportable for enterprises as well as providing tools to knock datasets into shape so they can feed into AI training runs. || EVIDENCE: Wang’s team brought over from Scale AI is one of the kernels of the Superintelligence Lab that Zuck &amp; Co have spent untold billions of dollars funding in the past year, bringing in fresh AI research talent and counterbalancing the loss of Yann LeCun, the long-time leader of the Facebook AI Research lab at New York University and one of the key researchers behind the development of the convolutional neural network more than four decades ago. || AFTER: (LeCun left FAIR a few weeks ago to start Advanced Machine Intelligence Labs, and has made no secret that he does not think the future of AI is GenAI LLMs.)</t>
         </is>
       </c>
-      <c r="T26" t="inlineStr"/>
-      <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr"/>
-      <c r="W26" t="inlineStr"/>
-      <c r="X26" t="inlineStr"/>
       <c r="Y26" t="inlineStr">
         <is>
           <t>person:yann_lecun</t>
@@ -4709,9 +4536,6 @@
       <c r="AK26" t="n">
         <v>0.5102440714836121</v>
       </c>
-      <c r="AL26" t="inlineStr"/>
-      <c r="AM26" t="inlineStr"/>
-      <c r="AN26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4776,7 +4600,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
           <t>Thus far, AMD has managed to unlock sizable gains through its ROCm stack since the launch of its MI300-series parts back in December.</t>
@@ -4797,11 +4620,6 @@
           <t>BEFORE: Speeds and feeds are great, but hardware is only as useful as the software that can harness it, and, for AMD, that’s the ROCm software stack. || EVIDENCE: If you’re not familiar, ROCm is to AMD’s Instinct GPU accelerators what CUDA is to Nvidia GPUs. || AFTER: The respective software suites are essential to tapping into their hardware platform’s full potential, and ROCm is a particularly big one encompassing everything from drivers, development tools, libraries, and APIs necessary for running compute workloads on AMD kit.</t>
         </is>
       </c>
-      <c r="T27" t="inlineStr"/>
-      <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr"/>
-      <c r="W27" t="inlineStr"/>
-      <c r="X27" t="inlineStr"/>
       <c r="Y27" t="inlineStr">
         <is>
           <t>technology:rocm</t>
@@ -4865,9 +4683,6 @@
       <c r="AK27" t="n">
         <v>0.5266782641410828</v>
       </c>
-      <c r="AL27" t="inlineStr"/>
-      <c r="AM27" t="inlineStr"/>
-      <c r="AN27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4932,7 +4747,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
         <is>
           <t>The platform’s NVLink bandwidth can top out at 130 TBps while networking speeds reach 14.4 TBps.</t>
@@ -4958,10 +4772,6 @@
           <t>BEFORE: The liquid-cooled DGX SuperPod with DGX GB300 systems consists of eight GB300 NVL72 platforms, amounting to 288 Grace CPUs, 576 Blackwell Ultra GPUs and 300 TB of fast memory that can produce 11.4 exaflops of FP4 computation. || EVIDENCE: The DGX SuperPod with DGX B300 systems, on the other hand, is pitched by Nvidia as a “ scalable, air-cooled architecture ” that will be offered as a new design for the company’s modular MGX server racks and enterprise data centers. || AFTER: Nvidia provided a major road map update in March, saying that the company plans to release a rack-scale architecture for AI data centers that will connect 576 next-generation GPUs in the second half of 2027.</t>
         </is>
       </c>
-      <c r="U28" t="inlineStr"/>
-      <c r="V28" t="inlineStr"/>
-      <c r="W28" t="inlineStr"/>
-      <c r="X28" t="inlineStr"/>
       <c r="Y28" t="inlineStr">
         <is>
           <t>product:dgx_superpod</t>
@@ -5102,7 +4912,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
           <t>Collaborations with Microsoft (for Azure distribution), Nvidia, and top European companies have further strengthened its growth trajectory.</t>
@@ -5123,11 +4932,6 @@
           <t>BEFORE: Its €600 million Series B in June 2024 pushed the valuation to nearly €6 billion, making it Europe’s highest-valued AI startup. || EVIDENCE: Major investors include General Catalyst, Andreessen Horowitz, Nvidia, Salesforce, IBM, and Microsoft, with Microsoft also partnering to distribute Mistral’s models through Azure. || AFTER: This robust financial backing and strategic partnerships have attracted prominent European clients like BNP Paribas, AXA, Stellantis, and CMA CGM, who value Mistral’s commitment to European data sovereignty and technical excellence.</t>
         </is>
       </c>
-      <c r="T29" t="inlineStr"/>
-      <c r="U29" t="inlineStr"/>
-      <c r="V29" t="inlineStr"/>
-      <c r="W29" t="inlineStr"/>
-      <c r="X29" t="inlineStr"/>
       <c r="Y29" t="inlineStr">
         <is>
           <t>org:salesforce</t>
@@ -5191,9 +4995,6 @@
       <c r="AK29" t="n">
         <v>0.7207024693489075</v>
       </c>
-      <c r="AL29" t="inlineStr"/>
-      <c r="AM29" t="inlineStr"/>
-      <c r="AN29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5258,7 +5059,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr">
         <is>
           <t>Liang Wenfeng, who founded the firm just two years ago, says his aim is ‘ not to lose money, nor to make huge profits’
@@ -5280,11 +5080,6 @@
           <t>BEFORE: Negative Sentiment: One market note also highlighted that Alibaba shares have lagged other major Chinese tech names this year, reflecting ongoing skepticism around Chinese internet stocks despite AI enthusiasm. || EVIDENCE: Here's why Alibaba, Tencent, Xiaomi stocks are falling amid the AI boom Analysts Set New Price || AFTER: TargetsA number of analysts have recently issued reports on BABA shares.</t>
         </is>
       </c>
-      <c r="T30" t="inlineStr"/>
-      <c r="U30" t="inlineStr"/>
-      <c r="V30" t="inlineStr"/>
-      <c r="W30" t="inlineStr"/>
-      <c r="X30" t="inlineStr"/>
       <c r="Y30" t="inlineStr">
         <is>
           <t>org:tencent</t>
@@ -5348,9 +5143,6 @@
       <c r="AK30" t="n">
         <v>0.547355055809021</v>
       </c>
-      <c r="AL30" t="inlineStr"/>
-      <c r="AM30" t="inlineStr"/>
-      <c r="AN30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5415,7 +5207,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
           <t>Learn more about the NVIDIA Vera Rubin platform.</t>
@@ -5441,10 +5232,6 @@
           <t>BEFORE: It was a message that he’s repeated this week at Nvidia’s GTC 2026 conference in San Jose, California. || EVIDENCE: For sure, there was been plenty of hardware talk during Huang’s keynote address during the show’s opening day, including platforms from Grace-Blackwell NVL72 to Vera-Rubin NVL72 to Nvidia’s plans for the Groq Language Processing Units (LPUs), not to mention storage systems and interconnects and the cloud business. || AFTER: But the overall focus of both the talk and the conference itself has been agentic AI, a market in which Nvidia is the dominant player, a position that Huang intends to keep and is willing spend a lot of money to ensure.</t>
         </is>
       </c>
-      <c r="U31" t="inlineStr"/>
-      <c r="V31" t="inlineStr"/>
-      <c r="W31" t="inlineStr"/>
-      <c r="X31" t="inlineStr"/>
       <c r="Y31" t="inlineStr">
         <is>
           <t>hardware:nvl72</t>
@@ -5616,10 +5403,26 @@
           <t>BEFORE: In November 2024 the company released its first version of Tülu 3, which had both 8- and 70-billion parameter versions. || EVIDENCE: At the time, Ai2 claimed the model was on par with the latest GPT-4 model from OpenAI, Anthropic’s Claude and Google’s Gemini. || AFTER: The big difference is that Tülu 3 is open-source.</t>
         </is>
       </c>
-      <c r="U32" t="inlineStr"/>
-      <c r="V32" t="inlineStr"/>
-      <c r="W32" t="inlineStr"/>
-      <c r="X32" t="inlineStr"/>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>sentence only lists Gemini and Claude as examples, no competition stated; also wrong entity:"Google" taken instead of "Gemini" - insufficent_context and entity_linking</t>
+        </is>
+      </c>
       <c r="Y32" t="inlineStr">
         <is>
           <t>model:claude</t>
@@ -5760,7 +5563,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr">
         <is>
           <t>(AP Photo/Ted S. Warren, File)
@@ -5783,11 +5585,21 @@
 Tech companies have long argued that “ fair use ” or “ fair dealing ” legal doctrines in the United States and United Kingdom allow them to train their AI systems on large troves of writings or images.</t>
         </is>
       </c>
-      <c r="T33" t="inlineStr"/>
-      <c r="U33" t="inlineStr"/>
-      <c r="V33" t="inlineStr"/>
-      <c r="W33" t="inlineStr"/>
-      <c r="X33" t="inlineStr"/>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>explicitly stated</t>
+        </is>
+      </c>
       <c r="Y33" t="inlineStr">
         <is>
           <t>org:getty</t>
@@ -5851,9 +5663,6 @@
       <c r="AK33" t="n">
         <v>0.6223466396331787</v>
       </c>
-      <c r="AL33" t="inlineStr"/>
-      <c r="AM33" t="inlineStr"/>
-      <c r="AN33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5918,7 +5727,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
         <is>
           <t>It also won’t be the last Chinese AI model to threaten the dominance of Silicon Valley giants — even as they, like OpenAI, raise more money than ever for their ambitions to develop artificial general intelligence (AGI), programs that outperform humans at most economically valuable work.</t>
@@ -5939,11 +5747,21 @@
           <t>BEFORE: Entrepreneur and commentator Arnaud Bertrand captured this dynamic, contrasting China’s frugal, decentralized innovation with the U.S. reliance on centralized, resource-intensive infrastructure: “ It’s about the world realizing that China has caught up — and in some areas overtaken — the U.S. in tech and innovation, despite efforts to prevent just that. ” || EVIDENCE: Indeed, yesterday another Chinese company, ByteDance, announced Doubao-1.5-pro, which Includes a “ Deep Thinking ” mode that surpasses OpenAI’s o1 on the AIME benchmark. || AFTER: Want to dive deeper into how DeepSeek-R1 is reshaping AI development?</t>
         </is>
       </c>
-      <c r="T34" t="inlineStr"/>
-      <c r="U34" t="inlineStr"/>
-      <c r="V34" t="inlineStr"/>
-      <c r="W34" t="inlineStr"/>
-      <c r="X34" t="inlineStr"/>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>explicitly stated</t>
+        </is>
+      </c>
       <c r="Y34" t="inlineStr">
         <is>
           <t>product:doubao_1_5_pro_2</t>
@@ -6007,9 +5825,6 @@
       <c r="AK34" t="n">
         <v>0.6558141708374023</v>
       </c>
-      <c r="AL34" t="inlineStr"/>
-      <c r="AM34" t="inlineStr"/>
-      <c r="AN34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -6107,10 +5922,21 @@
 Google released API pricing for Gemini 2.5 Pro, charging $ 1.25 per million input tokens and $ 10 per million output tokens for prompts up to 200,000 tokens and $ 2.50/ $ 15 per million input/output tokens for longer prompts. || EVIDENCE: The new model costs more than Google’s other AI offerings or competing models from OpenAI and DeepSeek, but remains cheaper than Anthropic’s Claude 3.7 Sonnet and OpenAI’s GPT-4.5. || AFTER: Developers responded positively to the pricing, marking an industry trend of increasing costs for flagship models.</t>
         </is>
       </c>
-      <c r="U35" t="inlineStr"/>
-      <c r="V35" t="inlineStr"/>
-      <c r="W35" t="inlineStr"/>
-      <c r="X35" t="inlineStr"/>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>explicitly stated</t>
+        </is>
+      </c>
       <c r="Y35" t="inlineStr">
         <is>
           <t>model:claude</t>
@@ -6251,7 +6077,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
         <is>
           <t>Microsoft also unveiled several new capabilities including Actions (which can complete tasks like booking reservations), Copilot Vision for mobile devices, Pages for content organization, AI-generated podcasts, shopping features, and its own implementation of Deep Research.</t>
@@ -6278,10 +6103,21 @@
           <t>BEFORE: Instead of listing out the steps, it did it right away which I did not want it to do. || EVIDENCE: In all fairness, Gemma 4 and Copilot are from different companies (Google and Microsoft) and since Copilot is built into Visual Studio Code, it is fair to assume that its actions strictly follows based on the settings you have in Visual Studio Code for Copilot. || AFTER: However, it is always nice to see Gemma 4 listing out the To-do list and asking the user to proceed.</t>
         </is>
       </c>
-      <c r="U36" t="inlineStr"/>
-      <c r="V36" t="inlineStr"/>
-      <c r="W36" t="inlineStr"/>
-      <c r="X36" t="inlineStr"/>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>explicitly stated</t>
+        </is>
+      </c>
       <c r="Y36" t="inlineStr">
         <is>
           <t>product:copilot</t>
@@ -6422,7 +6258,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
         <is>
           <t>GPU NVIDIA Installation
@@ -6449,11 +6284,26 @@
 Learn how to easily start using Ray on GKE by running a workload on a Ray cluster.</t>
         </is>
       </c>
-      <c r="T37" t="inlineStr"/>
-      <c r="U37" t="inlineStr"/>
-      <c r="V37" t="inlineStr"/>
-      <c r="W37" t="inlineStr"/>
-      <c r="X37" t="inlineStr"/>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>duplicate_or_noise</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>evidence is page boilerplate ("GenAI NVIDIA NeMo") + sentence about using GKE: nothing says NVIDIA developed GKE</t>
+        </is>
+      </c>
       <c r="Y37" t="inlineStr">
         <is>
           <t>platform:gke</t>
@@ -6517,9 +6367,6 @@
       <c r="AK37" t="n">
         <v>0.5383983254432678</v>
       </c>
-      <c r="AL37" t="inlineStr"/>
-      <c r="AM37" t="inlineStr"/>
-      <c r="AN37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6584,8 +6431,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr">
         <is>
           <t>A year after spending over $ 14 billion to bring in Alexandr Wang and a group of his top Scale AI engineers to revamp its artificial intelligence efforts, Meta is at least back on the map in AI, though it's still far behind OpenAI, Anthropic and Google in the market.</t>
@@ -6601,11 +6446,26 @@
           <t>EVIDENCE: Meta is debuting its first major artificial intelligence model since the costly hiring of Scale AI's Alexandr Wang nine months ago, as the Facebook parent aims to carve out a niche in a market that's being dominated by OpenAI, Anthropic and Google. || AFTER: Dubbed Muse Spark and originally code-named Avocado, the AI model announced Wednesday is the first from the company's new Muse series developed by Meta Superintelligence Labs, the AI unit that Wang oversees.</t>
         </is>
       </c>
-      <c r="T38" t="inlineStr"/>
-      <c r="U38" t="inlineStr"/>
-      <c r="V38" t="inlineStr"/>
-      <c r="W38" t="inlineStr"/>
-      <c r="X38" t="inlineStr"/>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>entity_linking</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>competition is between Meta and Google; Scale AI is only where the engineers came from</t>
+        </is>
+      </c>
       <c r="Y38" t="inlineStr">
         <is>
           <t>org:google</t>
@@ -6669,9 +6529,6 @@
       <c r="AK38" t="n">
         <v>0.6108084321022034</v>
       </c>
-      <c r="AL38" t="inlineStr"/>
-      <c r="AM38" t="inlineStr"/>
-      <c r="AN38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -6736,7 +6593,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr">
         <is>
           <t>More information can be found in our docs.</t>
@@ -6757,11 +6613,21 @@
           <t>BEFORE: You can unsubscribe at any time. || EVIDENCE: Cohere Labs Command R7B is an open weights research release of a 7B billion parameter model with advanced capabilities optimized for a variety of use cases including reasoning, summarization, question answering, and code. || AFTER: The model is trained to perform sophisticated tasks including Retrieval Augmented Generation (RAG) and tool use.</t>
         </is>
       </c>
-      <c r="T39" t="inlineStr"/>
-      <c r="U39" t="inlineStr"/>
-      <c r="V39" t="inlineStr"/>
-      <c r="W39" t="inlineStr"/>
-      <c r="X39" t="inlineStr"/>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>explicitly stated</t>
+        </is>
+      </c>
       <c r="Y39" t="inlineStr">
         <is>
           <t>model:command_r7b</t>
@@ -6825,9 +6691,6 @@
       <c r="AK39" t="n">
         <v>0.8057554364204407</v>
       </c>
-      <c r="AL39" t="inlineStr"/>
-      <c r="AM39" t="inlineStr"/>
-      <c r="AN39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -6892,7 +6755,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr">
         <is>
           <t>He directly challenges the popular interpretation:
@@ -6919,10 +6781,21 @@
           <t>BEFORE: It also offers low, medium and high reasoning effort settings, so users can tailor the model to both basic and more challenging problems. || EVIDENCE: Claude 3.7 Sonnet is one of the latest large language models released by Anthropic, an AI research and development company that counts Google and Amazon among its investors. || AFTER: Claude 3.7 Sonnet features a standard and extended thinking mode, with the latter giving it the ability to reflect before responding.</t>
         </is>
       </c>
-      <c r="U40" t="inlineStr"/>
-      <c r="V40" t="inlineStr"/>
-      <c r="W40" t="inlineStr"/>
-      <c r="X40" t="inlineStr"/>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>explicitly stated</t>
+        </is>
+      </c>
       <c r="Y40" t="inlineStr">
         <is>
           <t>model:sonnet</t>
@@ -7063,7 +6936,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
           <t>To show the prowess of its work, DeepSeek also used R1 to distill six Llama and Qwen models, taking their performance to new levels.</t>
@@ -7089,10 +6961,26 @@
           <t>BEFORE: OpenAI recently responded with Operator, its own foray into using vision and language models to control computers. || EVIDENCE: Results: UI-TARS matched or outperformed Claude 3.5 Sonnet with computer use, GPT-4o with various computer use frameworks, and the Aguvis framework with its native model on 11 benchmarks. || AFTER: On OSWorld, which asks models to perform tasks using a variety of real-world applications and operating systems, UI-TARS successfully completed 22.7 percent of the tasks in 15 steps, whereas Claude 3.5 Sonnet with computer use completed 14.9 percent, GPT-4o with Aguvis 17 percent, and Aguvis with its native model 10.3 percent.</t>
         </is>
       </c>
-      <c r="U41" t="inlineStr"/>
-      <c r="V41" t="inlineStr"/>
-      <c r="W41" t="inlineStr"/>
-      <c r="X41" t="inlineStr"/>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>entity_linking</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>Qwen-1.5B that outperforms GPT and Sonnet, GPT and Sonnet are not compared with each other</t>
+        </is>
+      </c>
       <c r="Y41" t="inlineStr">
         <is>
           <t>model:gpt_4o_2</t>
@@ -7233,7 +7121,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
         <is>
           <t>The chipmaker lost close to $ 600 billion in market cap, the biggest drop for any company on a single day in U.S. history.</t>
@@ -7254,11 +7141,26 @@
           <t>BEFORE: DeepSeek-R1 released on Jan 20th, 2025 sent shockwaves through the stock market, particularly impacting technology companies that are heavily invested in AI. || EVIDENCE: Major US tech companies like NVIDIA, Broadcom, and AMD saw significant drops in their stock prices, with NVIDIA experiencing a record-one-day market capitalization loss of over $ 500 billion. || AFTER: This disruption was caused due to DeepSeek-R1’s competitive performance and significantly lower cost which challenged the dominance of existing players like OpenAI and NVIDIA.</t>
         </is>
       </c>
-      <c r="T42" t="inlineStr"/>
-      <c r="U42" t="inlineStr"/>
-      <c r="V42" t="inlineStr"/>
-      <c r="W42" t="inlineStr"/>
-      <c r="X42" t="inlineStr"/>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>insufficient_context</t>
+        </is>
+      </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>US refers to stock market not headquarters</t>
+        </is>
+      </c>
       <c r="Y42" t="inlineStr">
         <is>
           <t>org:broadcom</t>
@@ -7322,9 +7224,6 @@
       <c r="AK42" t="n">
         <v>0.516190230846405</v>
       </c>
-      <c r="AL42" t="inlineStr"/>
-      <c r="AM42" t="inlineStr"/>
-      <c r="AN42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -7389,7 +7288,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr">
         <is>
           <t>This device isn’t just for gaming.</t>
@@ -7410,11 +7308,21 @@
           <t>BEFORE: Meta is positioning the Quest 4 as a versatile tool for multiple applications, including fitness and productivity. || EVIDENCE: With enhanced fitness-tracking capabilities and a growing library of wellness apps, the Quest 4 is Meta’s attempt to push VR beyond its traditional entertainment boundaries. || AFTER: Mark Zuckerberg highlighted that VR has the potential to revolutionize fitness by making exercise more engaging through immersive environments and real-time tracking.</t>
         </is>
       </c>
-      <c r="T43" t="inlineStr"/>
-      <c r="U43" t="inlineStr"/>
-      <c r="V43" t="inlineStr"/>
-      <c r="W43" t="inlineStr"/>
-      <c r="X43" t="inlineStr"/>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>explicitly stated</t>
+        </is>
+      </c>
       <c r="Y43" t="inlineStr">
         <is>
           <t>product:quest_4</t>
@@ -7478,9 +7386,6 @@
       <c r="AK43" t="n">
         <v>0.6226887702941895</v>
       </c>
-      <c r="AL43" t="inlineStr"/>
-      <c r="AM43" t="inlineStr"/>
-      <c r="AN43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -7575,10 +7480,26 @@
           <t>BEFORE: Indeed, the launch of DeepSeek-R1 appears to be taking the generative AI industry into a new era of brinkmanship, where the wealthiest companies with the largest models may no longer win by default. || EVIDENCE: DeepSeek-R1 is an open source language model developed by DeepSeek, a Chinese startup founded in 2023 by Liang Wenfeng, who also co-founded quantitative hedge fund High-Flyer. || AFTER: The company reportedly grew out of High-Flyer’s AI research unit to focus on developing large language models that achieve artificial general intelligence (AGI) — a benchmark where AI is able to match human intellect, which OpenAI and other top AI companies are also working towards.</t>
         </is>
       </c>
-      <c r="U44" t="inlineStr"/>
-      <c r="V44" t="inlineStr"/>
-      <c r="W44" t="inlineStr"/>
-      <c r="X44" t="inlineStr"/>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>entity_linking</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>founder is Liang not High-Flyer; High-Flyer is another company he founded</t>
+        </is>
+      </c>
       <c r="Y44" t="inlineStr">
         <is>
           <t>org:deepseek</t>
@@ -7719,7 +7640,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr">
         <is>
           <t>(The company previously released a 2-billion-parameter model trained in 10 Indian languages, called Sarvam-1.)</t>
@@ -7745,10 +7665,21 @@
           <t>BEFORE: In late May, Sarvam AI unveiled Sarvam‑M, a 24-billion-parameter multilingual LLM fine-tuned for 10 Indian languages and built on top of Mistral Small, an efficient model developed by the French company Mistral AI. || EVIDENCE: Sarvam’s cofounder Vivek Raghavan called the model “ an important stepping stone on our journey to build sovereign AI for India. ” || AFTER: But its download numbers were underwhelming, with only 300 in the first two days.</t>
         </is>
       </c>
-      <c r="U45" t="inlineStr"/>
-      <c r="V45" t="inlineStr"/>
-      <c r="W45" t="inlineStr"/>
-      <c r="X45" t="inlineStr"/>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>AMBIGUOUS</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>Sarvam is part of the IndiaAI mission, which suggests an Indian company, but HQ is not stated</t>
+        </is>
+      </c>
       <c r="Y45" t="inlineStr">
         <is>
           <t>org:sarvam</t>
@@ -7889,7 +7820,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr">
         <is>
           <t>This approach has challenged conventional convolutional neural networks (CNNs), offering a new perspective on processing visual information.</t>
@@ -7915,10 +7845,21 @@
           <t>BEFORE: The impact of the GPT series goes beyond technological achievements; it has ignited discussions regarding AI’s potential to replicate human creativity with AI-generated content, as well as ethical implications shaping the future landscape of human-AI interactions. || EVIDENCE: BERT (Bidirectional Encoder Representations from Transformers) by Google introduces an approach for leveraging context in language models. || AFTER: BERT uses a bidirectional attention mechanism that considers both the preceding and following context of each word in a sentence.</t>
         </is>
       </c>
-      <c r="U46" t="inlineStr"/>
-      <c r="V46" t="inlineStr"/>
-      <c r="W46" t="inlineStr"/>
-      <c r="X46" t="inlineStr"/>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="X46" t="inlineStr">
+        <is>
+          <t>support_2_context explicilty state it</t>
+        </is>
+      </c>
       <c r="Y46" t="inlineStr">
         <is>
           <t>technology:bidirectional_encoder_representations_from_transformers</t>
@@ -8059,8 +8000,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr"/>
       <c r="Q47" t="inlineStr">
         <is>
           <t>When DeepSeek released its R1 model this January, it wasn’t just another AI announcement.</t>
@@ -8081,10 +8020,21 @@
           <t>BEFORE: Both usually take place in data centers, where they require lots of energy to run chips and cool servers. || EVIDENCE: On the training side for its R1 model, DeepSeek’s team improved what’s called a “ mixture of experts ” technique, in which only a portion of a model’s billions of parameters—the “ knobs ” a model uses to form better answers—are turned on at a given time during training. || AFTER: More notably, they improved reinforcement learning, where a model’s outputs are scored and then used to make it better.</t>
         </is>
       </c>
-      <c r="U47" t="inlineStr"/>
-      <c r="V47" t="inlineStr"/>
-      <c r="W47" t="inlineStr"/>
-      <c r="X47" t="inlineStr"/>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="X47" t="inlineStr">
+        <is>
+          <t>explicitly stated</t>
+        </is>
+      </c>
       <c r="Y47" t="inlineStr">
         <is>
           <t>model:r1_model</t>
@@ -8225,7 +8175,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr">
         <is>
           <t>LiteLLM is a great starting point for developers who want a simple way to integrate multiple LLMs, but as projects grow, infrastructure needs become more complex.</t>
@@ -8246,11 +8195,26 @@
           <t>BEFORE: As the GenAI ecosystem matures, it's worth evaluating platforms that align with how you build, monitor, and grow your LLM-powered products. || EVIDENCE: While tools like Portkey and Helicone offer gateway features, TrueFoundry stands out as the premier LiteLLM alternative for high-performance needs. || AFTER: Unlike LiteLLM, which can introduce significant latency, TrueFoundry’s AI Gateway operates with a minimal ~3–4ms overhead and handles 350+ RPS on a single vCPU.</t>
         </is>
       </c>
-      <c r="T48" t="inlineStr"/>
-      <c r="U48" t="inlineStr"/>
-      <c r="V48" t="inlineStr"/>
-      <c r="W48" t="inlineStr"/>
-      <c r="X48" t="inlineStr"/>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>insufficient_context</t>
+        </is>
+      </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>listed together as alternatives; no competition</t>
+        </is>
+      </c>
       <c r="Y48" t="inlineStr">
         <is>
           <t>org:truefoundry</t>
@@ -8314,9 +8278,6 @@
       <c r="AK48" t="n">
         <v>0.5730122923851013</v>
       </c>
-      <c r="AL48" t="inlineStr"/>
-      <c r="AM48" t="inlineStr"/>
-      <c r="AN48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -8381,7 +8342,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr">
         <is>
           <t>According to China's Top 10 AI applications ranking, general AI assistants Doubao and DeepSeek have emerged as dominant portals.</t>
@@ -8407,10 +8367,21 @@
           <t>BEFORE: Chinese media outlet 36Kr reported that Minimax’s revenue in 2024 was around $ 70 million, making it one of the most successful consumer-facing Chinese AI startups in the global market. || EVIDENCE: Moonshot is best known for building Kimi, the second-most-popular AI chatbot in China, just after ByteDance’s Doubao, with over 13 million users. || AFTER: Released in 2023, Kimi supports input lengths of over 200,000 characters, making it a popular choice among students, white-collar workers, and others who routinely have to work with long chunks of text.</t>
         </is>
       </c>
-      <c r="U49" t="inlineStr"/>
-      <c r="V49" t="inlineStr"/>
-      <c r="W49" t="inlineStr"/>
-      <c r="X49" t="inlineStr"/>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>direct market competition</t>
+        </is>
+      </c>
       <c r="Y49" t="inlineStr">
         <is>
           <t>model:kimi</t>
@@ -8576,11 +8547,26 @@
           <t>BEFORE: At Computex, AMD unveiled plans to release a new Instinct data center GPU, the MI325X, later this year with significantly greater high-bandwidth memory than its MI300X chip or Nvidia’s H200, enabling servers to handle larger generative AI models than before. || EVIDENCE: The MI325X is set to arrive in systems from Dell, Lenovo, Supermicro, Hewlett Packard Enterprise, Gigabyte, Eviden and several other server vendors starting in the first quarter of next year, according to AMD. || AFTER: AMD unveiled the details as part of a newly disclosed plan to release a new data center GPU every year starting with the CDNA 3-based MI325X. In an extended road map, AMD said it will then debut in 2025 the MI350 series, which will use its CDNA 4 architecture to provide increased compute performance and “ memory leadership. ”</t>
         </is>
       </c>
-      <c r="T50" t="inlineStr"/>
-      <c r="U50" t="inlineStr"/>
-      <c r="V50" t="inlineStr"/>
-      <c r="W50" t="inlineStr"/>
-      <c r="X50" t="inlineStr"/>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>insufficient_context</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>listed together as sellers; no competition or comparison is stated</t>
+        </is>
+      </c>
       <c r="Y50" t="inlineStr">
         <is>
           <t>org:dell</t>
@@ -8644,9 +8630,6 @@
       <c r="AK50" t="n">
         <v>0.543927788734436</v>
       </c>
-      <c r="AL50" t="inlineStr"/>
-      <c r="AM50" t="inlineStr"/>
-      <c r="AN50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -8711,7 +8694,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr">
         <is>
           <t>Google signed its first publisher deal with the Associated Press in January 2025.</t>
@@ -8732,11 +8714,21 @@
           <t>BEFORE: This guide will take you through how to use both of ChatGPT's voice modes. || EVIDENCE: Amazon has to overcome'several technical hurdles ' because it can roll out the new Alexa, according to The Financial Times. || AFTER: On Monday, British Minister Keir Starmer announced a new AI Opportunities Action Plan.</t>
         </is>
       </c>
-      <c r="T51" t="inlineStr"/>
-      <c r="U51" t="inlineStr"/>
-      <c r="V51" t="inlineStr"/>
-      <c r="W51" t="inlineStr"/>
-      <c r="X51" t="inlineStr"/>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>explicitly stated</t>
+        </is>
+      </c>
       <c r="Y51" t="inlineStr">
         <is>
           <t>model:alexa</t>
@@ -8800,9 +8792,6 @@
       <c r="AK51" t="n">
         <v>0.6422073841094971</v>
       </c>
-      <c r="AL51" t="inlineStr"/>
-      <c r="AM51" t="inlineStr"/>
-      <c r="AN51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -8867,7 +8856,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr">
         <is>
           <t>Moreover, if the cloud partnership terminates, Amazon’s remaining $ 35 billion commitment will die with it.</t>
@@ -8893,10 +8881,26 @@
           <t>BEFORE: And then obviously they have this announced commitment to build even more data centers. || EVIDENCE: And then obviously there’s that weird circular financing dance that’s happening in AI, where NVIDIA invests in OpenAI and OpenAI invests in CoreWeave, and then OpenAI buys NVIDIA chips. || AFTER: I mean, people are paying attention.</t>
         </is>
       </c>
-      <c r="U52" t="inlineStr"/>
-      <c r="V52" t="inlineStr"/>
-      <c r="W52" t="inlineStr"/>
-      <c r="X52" t="inlineStr"/>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>reversed_direction</t>
+        </is>
+      </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>Nvidia invested in OpenAI</t>
+        </is>
+      </c>
       <c r="Y52" t="inlineStr">
         <is>
           <t>org:openai</t>
@@ -9037,7 +9041,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O53" t="inlineStr"/>
       <c r="P53" t="inlineStr">
         <is>
           <t>This approach allows it to excel in tasks requiring advanced reasoning, logical problem-solving, and adaptability to complex scenarios.</t>
@@ -9058,11 +9061,21 @@
           <t>BEFORE: Multi-head Latent Attention is a variation on multi-head attention that was introduced by DeepSeek in their V2 paper. || EVIDENCE: According to this post, while previous multi-head attention techniques were considered a tradeoff, insofar as you reduce model quality to get better scale in large model training, DeepSeek says that MLA not only allows scale, it also improves the model. || AFTER: We’re looking forward to digging deeper into this.</t>
         </is>
       </c>
-      <c r="T53" t="inlineStr"/>
-      <c r="U53" t="inlineStr"/>
-      <c r="V53" t="inlineStr"/>
-      <c r="W53" t="inlineStr"/>
-      <c r="X53" t="inlineStr"/>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="X53" t="inlineStr">
+        <is>
+          <t>explicitly stated</t>
+        </is>
+      </c>
       <c r="Y53" t="inlineStr">
         <is>
           <t>standard:mla</t>
@@ -9126,9 +9139,6 @@
       <c r="AK53" t="n">
         <v>0.6532100439071655</v>
       </c>
-      <c r="AL53" t="inlineStr"/>
-      <c r="AM53" t="inlineStr"/>
-      <c r="AN53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -9193,7 +9203,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr">
         <is>
           <t>In the code above, the string "gemma #  xxxxxxx" specifies a preset version and parameter size for Gemma.</t>
@@ -9214,11 +9223,21 @@
           <t>BEFORE: It is also trained on over 100 languages, making it versatile and capable of generating high-quality embeddings for a wide range of global applications. || EVIDENCE: EmbeddingGemma’s model weights are available on HuggingFace, Kaggle, and VertexAI. || AFTER: It seamlessly integrates with on-device tools such as transformers.js, MLX, llama.cpp, LiteRT, Ollama, LMStudio, etc.</t>
         </is>
       </c>
-      <c r="T54" t="inlineStr"/>
-      <c r="U54" t="inlineStr"/>
-      <c r="V54" t="inlineStr"/>
-      <c r="W54" t="inlineStr"/>
-      <c r="X54" t="inlineStr"/>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="X54" t="inlineStr">
+        <is>
+          <t>explicitly stated</t>
+        </is>
+      </c>
       <c r="Y54" t="inlineStr">
         <is>
           <t>model:gemma</t>
@@ -9282,9 +9301,6 @@
       <c r="AK54" t="n">
         <v>0.7573210000991821</v>
       </c>
-      <c r="AL54" t="inlineStr"/>
-      <c r="AM54" t="inlineStr"/>
-      <c r="AN54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -9349,7 +9365,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O55" t="inlineStr"/>
       <c r="P55" t="inlineStr">
         <is>
           <t>In November 2024, Robinhood announced the $ 300 million acquisition of TradePMR, a custodial and portfolio management platform specializing in services for Registered Investment Advisors.</t>
@@ -9370,11 +9385,26 @@
           <t>BEFORE: Despite the recent dip, Robinhood shares have soared 75.1% in the past three months, significantly outperforming the industry’s rally of 18.1%. || EVIDENCE: Further, in contrast, its peers – SCHW and LPLA – are up just 15% and 35.7%, respectively, in the same time frame. || AFTER: Additionally, over the past month, the Zacks Consensus Estimate for 2024 and 2025 earnings has moved upward.</t>
         </is>
       </c>
-      <c r="T55" t="inlineStr"/>
-      <c r="U55" t="inlineStr"/>
-      <c r="V55" t="inlineStr"/>
-      <c r="W55" t="inlineStr"/>
-      <c r="X55" t="inlineStr"/>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>entity_linking</t>
+        </is>
+      </c>
+      <c r="X55" t="inlineStr">
+        <is>
+          <t>"the company" compete with LPLA and SCHW; they're only listed together</t>
+        </is>
+      </c>
       <c r="Y55" t="inlineStr">
         <is>
           <t>org:lpla</t>
@@ -9438,9 +9468,6 @@
       <c r="AK55" t="n">
         <v>0.5848894119262695</v>
       </c>
-      <c r="AL55" t="inlineStr"/>
-      <c r="AM55" t="inlineStr"/>
-      <c r="AN55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -9505,7 +9532,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr">
         <is>
           <t>The crunch has forced companies like DeepSeek to get creative.</t>
@@ -9526,11 +9552,26 @@
           <t>BEFORE: That’s about $ 11.34 m/week. || EVIDENCE: In DeepSeek’s case, it appears they could have used GPUs that their hedge fund backer High-Flyer had acquired earlier for high-frequency trading purposes. || AFTER: There are a number of sophisticated ways in which DeepSeek modified the model architecture, training techniques and data to get the most out of the limited hardware available to them.</t>
         </is>
       </c>
-      <c r="T56" t="inlineStr"/>
-      <c r="U56" t="inlineStr"/>
-      <c r="V56" t="inlineStr"/>
-      <c r="W56" t="inlineStr"/>
-      <c r="X56" t="inlineStr"/>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>entity_linking</t>
+        </is>
+      </c>
+      <c r="X56" t="inlineStr">
+        <is>
+          <t>High-flyer acquired chips not DeepSeek itself</t>
+        </is>
+      </c>
       <c r="Y56" t="inlineStr">
         <is>
           <t>org:deepseek</t>
@@ -9594,9 +9635,6 @@
       <c r="AK56" t="n">
         <v>0.7170218825340271</v>
       </c>
-      <c r="AL56" t="inlineStr"/>
-      <c r="AM56" t="inlineStr"/>
-      <c r="AN56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -9661,8 +9699,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O57" t="inlineStr"/>
-      <c r="P57" t="inlineStr"/>
       <c r="Q57" t="inlineStr">
         <is>
           <t>Elon Musk’s artificial intelligence startup xAI has unveiled Grok 3, its latest AI model that the company claims outperforms leading competitors across key technical benchmarks.</t>
@@ -9683,10 +9719,21 @@
           <t>BEFORE: Trained through reinforcement learning, DeepSeek-R1 showcases extensive context and chain-of-thought reasoning to tackle complex subjects and situations. || EVIDENCE: Developed by Elon Musk’s AI company xAI, Grok 3 shares the same name as the Grok chatbot it powers. || AFTER: Grok 3 is another model trained with reinforcement learning, so it can evaluate its processes, fix its mistakes and adjust its performance over time.</t>
         </is>
       </c>
-      <c r="U57" t="inlineStr"/>
-      <c r="V57" t="inlineStr"/>
-      <c r="W57" t="inlineStr"/>
-      <c r="X57" t="inlineStr"/>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="X57" t="inlineStr">
+        <is>
+          <t>explicitly stated</t>
+        </is>
+      </c>
       <c r="Y57" t="inlineStr">
         <is>
           <t>product:grok_3</t>
@@ -9827,7 +9874,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr">
         <is>
           <t>The other major architectural component in DeepSeek worth highlighting is its use of Mixture-of-Experts (MoE) layers.</t>
@@ -9854,10 +9900,21 @@
 And finally, and perhaps most importantly, on January 20, DeepSeek rolled out its DeepSeek-R1 model, which adds two more reinforcement learning stages and two supervised fine tuning stages to enhance the model’s reasoning capabilities.</t>
         </is>
       </c>
-      <c r="U58" t="inlineStr"/>
-      <c r="V58" t="inlineStr"/>
-      <c r="W58" t="inlineStr"/>
-      <c r="X58" t="inlineStr"/>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="X58" t="inlineStr">
+        <is>
+          <t>explicitly stated</t>
+        </is>
+      </c>
       <c r="Y58" t="inlineStr">
         <is>
           <t>architecture:mixture_of_experts</t>
@@ -9998,7 +10055,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr">
         <is>
           <t>Gemini 3.1 Pro Preview is the basis of recent performance gains by Gemini 3 Deep Think, a specialized reasoning mode separate from the three reasoning levels available via API.</t>
@@ -10019,11 +10075,21 @@
           <t>BEFORE: Google updated its flagship Gemini model, topping several benchmarks while undercutting competitors on performance per dollar. || EVIDENCE: What’s new: Google launched Gemini 3.1 Pro Preview at the same price as its predecessor Gemini 3 Pro Preview. || AFTER: Gemini 3.1 Pro Preview is the basis of recent performance gains by Gemini 3 Deep Think, a specialized reasoning mode separate from the three reasoning levels available via API.</t>
         </is>
       </c>
-      <c r="T59" t="inlineStr"/>
-      <c r="U59" t="inlineStr"/>
-      <c r="V59" t="inlineStr"/>
-      <c r="W59" t="inlineStr"/>
-      <c r="X59" t="inlineStr"/>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="X59" t="inlineStr">
+        <is>
+          <t>stated in support_2_context</t>
+        </is>
+      </c>
       <c r="Y59" t="inlineStr">
         <is>
           <t>product:gemini_3_1_pro_preview</t>
@@ -10087,9 +10153,6 @@
       <c r="AK59" t="n">
         <v>0.6289657354354858</v>
       </c>
-      <c r="AL59" t="inlineStr"/>
-      <c r="AM59" t="inlineStr"/>
-      <c r="AN59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -10154,7 +10217,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr">
         <is>
           <t>It remains to be seen whether the current threshold strikes the right balance.</t>
@@ -10175,11 +10237,21 @@
           <t>BEFORE: The team compared the Hunyuan-Large models to four open source models and their instruction-tuned versions: Llama 3.1 70B, Llama 3.1 405B, and the MoE models Mixtral-8x22B and DeepSeek-V2. || EVIDENCE: Why it matters: Hunyuan-Large generally outperforms Llama 405B, achieving the performance of a 405 billion parameter model while computing only 52 billion parameters. || AFTER: That’s a significantly lower processing requirement, and the model is free for many purposes.</t>
         </is>
       </c>
-      <c r="T60" t="inlineStr"/>
-      <c r="U60" t="inlineStr"/>
-      <c r="V60" t="inlineStr"/>
-      <c r="W60" t="inlineStr"/>
-      <c r="X60" t="inlineStr"/>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="X60" t="inlineStr">
+        <is>
+          <t>explicitly stated</t>
+        </is>
+      </c>
       <c r="Y60" t="inlineStr">
         <is>
           <t>model:hunyuan</t>
@@ -10243,9 +10315,6 @@
       <c r="AK60" t="n">
         <v>0.7400286197662354</v>
       </c>
-      <c r="AL60" t="inlineStr"/>
-      <c r="AM60" t="inlineStr"/>
-      <c r="AN60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -10310,7 +10379,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O61" t="inlineStr"/>
       <c r="P61" t="inlineStr">
         <is>
           <t>The adoption of open source LLMs shows distinct regional and industry-specific patterns.</t>
@@ -10331,11 +10399,21 @@
           <t>BEFORE: SAP, another business app giant, announced comprehensive open source LLM support through its Joule AI copilot, while ServiceNow enabled both open and closed LLM integration for workflow automation in areas like customer service and IT support. || EVIDENCE: “ I think open models will ultimately win out, ” says Oracle’s EVP of AI and Data Management Services, Greg Pavlik. || AFTER: The ability to modify models and experiment, especially in vertical domains, combined with favorable cost, is proving compelling for enterprise customers, he said.</t>
         </is>
       </c>
-      <c r="T61" t="inlineStr"/>
-      <c r="U61" t="inlineStr"/>
-      <c r="V61" t="inlineStr"/>
-      <c r="W61" t="inlineStr"/>
-      <c r="X61" t="inlineStr"/>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>Reviewer_B</t>
+        </is>
+      </c>
+      <c r="X61" t="inlineStr">
+        <is>
+          <t>explicitly stated</t>
+        </is>
+      </c>
       <c r="Y61" t="inlineStr">
         <is>
           <t>person:greg_pavlik</t>
@@ -10399,9 +10477,6 @@
       <c r="AK61" t="n">
         <v>0.7015882730484009</v>
       </c>
-      <c r="AL61" t="inlineStr"/>
-      <c r="AM61" t="inlineStr"/>
-      <c r="AN61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -10466,7 +10541,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O62" t="inlineStr"/>
       <c r="P62" t="inlineStr">
         <is>
           <t>Offline capability.</t>
@@ -10488,11 +10562,26 @@
           <t>BEFORE: But for the tasks that actually matter to most people’s lives (agricultural advisories, legal services, medical triage, language preservation) they can be almost as effective as models costing a thousand times more to run. || EVIDENCE: The most compelling example I’ve encountered is the Saving Voices Project, a nonprofit founded by Arjuna Sathiaseelan, who is also the chief technology officer of the Frugal AI Hub at Cambridge University. || AFTER: The project recently built a custom speech AI system for the Soliga tribe in southern India.</t>
         </is>
       </c>
-      <c r="T62" t="inlineStr"/>
-      <c r="U62" t="inlineStr"/>
-      <c r="V62" t="inlineStr"/>
-      <c r="W62" t="inlineStr"/>
-      <c r="X62" t="inlineStr"/>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
+      <c r="W62" t="inlineStr">
+        <is>
+          <t>entity_linking</t>
+        </is>
+      </c>
+      <c r="X62" t="inlineStr">
+        <is>
+          <t>The founder relationship refers to Saving Voices Project. Support 2 identifies him as CTO of Frugal AI Hub, not its founder.</t>
+        </is>
+      </c>
       <c r="Y62" t="inlineStr">
         <is>
           <t>org:frugal_ai_hub</t>
@@ -10556,9 +10645,6 @@
       <c r="AK62" t="n">
         <v>0.6185426712036133</v>
       </c>
-      <c r="AL62" t="inlineStr"/>
-      <c r="AM62" t="inlineStr"/>
-      <c r="AN62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -10623,8 +10709,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O63" t="inlineStr"/>
-      <c r="P63" t="inlineStr"/>
       <c r="Q63" t="inlineStr">
         <is>
           <t>We post-trained NVIDIA Nemotron 3.5 Lightning for legal and healthcare in a few hours on a single node.</t>
@@ -10645,10 +10729,26 @@
           <t>BEFORE: This write-up covers post-training for enterprise domains. || EVIDENCE: EAGLE-3 speculative decoding for NVIDIA Nemotron 3.5 Lightning is its companion, and the two are submitted together. || AFTER: The adapters were trained and evaluated on Thoughtworks-operated AWS instances, and no corpus or generation left the node.</t>
         </is>
       </c>
-      <c r="U63" t="inlineStr"/>
-      <c r="V63" t="inlineStr"/>
-      <c r="W63" t="inlineStr"/>
-      <c r="X63" t="inlineStr"/>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
+      <c r="W63" t="inlineStr">
+        <is>
+          <t>entity_boundary</t>
+        </is>
+      </c>
+      <c r="X63" t="inlineStr">
+        <is>
+          <t>The evidence identifies NVIDIA Nemotron 3.5 Lightning. Lightning alone is an incomplete and ambiguous model name.</t>
+        </is>
+      </c>
       <c r="Y63" t="inlineStr">
         <is>
           <t>product:lightning</t>
@@ -10789,7 +10889,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O64" t="inlineStr"/>
       <c r="P64" t="inlineStr">
         <is>
           <t>Codex writes features, answers codebase questions, fixes bugs, and proposes pull requests, with each task running in its own isolated cloud environment preloaded with the user’s repository.</t>
@@ -10810,11 +10909,17 @@
           <t>BEFORE: In any case, the muted response to GPT-4.5 and Llama 4 (non-reasoning) models suggests we are approaching the limits of what scaling model size and data alone can achieve. || EVIDENCE: However, OpenAI's recent release of the o3 reasoning model demonstrates there is still considerable room for improvement when investing compute strategically, specifically via reinforcement learning methods tailored for reasoning tasks. || AFTER: (According to OpenAI staff during the recent livestream, o3 used 10× more training compute compared to o1.)</t>
         </is>
       </c>
-      <c r="T64" t="inlineStr"/>
-      <c r="U64" t="inlineStr"/>
-      <c r="V64" t="inlineStr"/>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
       <c r="W64" t="inlineStr"/>
-      <c r="X64" t="inlineStr"/>
       <c r="Y64" t="inlineStr">
         <is>
           <t>model:o3_reasoning_model</t>
@@ -10878,9 +10983,6 @@
       <c r="AK64" t="n">
         <v>0.7039905786514282</v>
       </c>
-      <c r="AL64" t="inlineStr"/>
-      <c r="AM64" t="inlineStr"/>
-      <c r="AN64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -10970,11 +11072,17 @@
           <t>BEFORE: This funding round was co-led by Cyber Fund, a premier and forward-thinking investment firm and creators of Lido and P2P.org, and Arche Capital, a venture capital firm co-founded by respected early-stage investors Vanessa Grellet and William Wolf. || EVIDENCE: The round was also backed by several other prominent investors, such as Seed Club Ventures, a Venture DAO backing early-stage founders and the first investor in Stability AI, the company behind Stable Diffusion, the widely successful open-source AI image generation model. || AFTER: Richard Blythman, Chief Scientific Officer and Co-Founder of Naptha AI said: “ The future of AI isn’t just about more powerful models; it’s about intelligent collaboration between diverse networks of agents.</t>
         </is>
       </c>
-      <c r="T65" t="inlineStr"/>
-      <c r="U65" t="inlineStr"/>
-      <c r="V65" t="inlineStr"/>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
       <c r="W65" t="inlineStr"/>
-      <c r="X65" t="inlineStr"/>
       <c r="Y65" t="inlineStr">
         <is>
           <t>org:seed_club_ventures</t>
@@ -11038,9 +11146,6 @@
       <c r="AK65" t="n">
         <v>0.6891469359397888</v>
       </c>
-      <c r="AL65" t="inlineStr"/>
-      <c r="AM65" t="inlineStr"/>
-      <c r="AN65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -11105,7 +11210,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O66" t="inlineStr"/>
       <c r="P66" t="inlineStr">
         <is>
           <t>It follows that the rate that LLM providers charge to use them will continue to drop as well.</t>
@@ -11131,10 +11235,17 @@
           <t>BEFORE: The company’s GenSRF (security, risk and fraud assessment) system, part of its “ GenOS ” operating system, monitors about 100 dimensions of trust and safety. || EVIDENCE: “ We have a committee that reviews LLMs and makes sure its standards are consistent with the company’s principles, ” Intuit’s Srivastava explains. || AFTER: However, he said these reviews of open models are no different than the ones the company makes for closed-sourced models.</t>
         </is>
       </c>
-      <c r="U66" t="inlineStr"/>
-      <c r="V66" t="inlineStr"/>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
       <c r="W66" t="inlineStr"/>
-      <c r="X66" t="inlineStr"/>
       <c r="Y66" t="inlineStr">
         <is>
           <t>person:ashok_srivastava</t>
@@ -11275,8 +11386,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O67" t="inlineStr"/>
-      <c r="P67" t="inlineStr"/>
       <c r="Q67" t="inlineStr">
         <is>
           <t>Ant Group releases Ling-2.5-1T and Ring-2.5-1T open-source AI models, advancing trillion-parameter reasoning and multimodal systems across its Ling family.</t>
@@ -11292,11 +11401,17 @@
           <t>BEFORE: Efficiency gains appear central to the update. || EVIDENCE: Ant Group reported that Ling-2.5-1T matches the performance of frontier reasoning models on the AIME 2026 benchmark while using substantially fewer tokens. || AFTER: Comparable systems typically require between 15,000 and 23,000 tokens for similar results.</t>
         </is>
       </c>
-      <c r="T67" t="inlineStr"/>
-      <c r="U67" t="inlineStr"/>
-      <c r="V67" t="inlineStr"/>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
       <c r="W67" t="inlineStr"/>
-      <c r="X67" t="inlineStr"/>
       <c r="Y67" t="inlineStr">
         <is>
           <t>model:ling_2_5_1t</t>
@@ -11360,9 +11475,6 @@
       <c r="AK67" t="n">
         <v>0.6956205368041992</v>
       </c>
-      <c r="AL67" t="inlineStr"/>
-      <c r="AM67" t="inlineStr"/>
-      <c r="AN67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -11427,7 +11539,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O68" t="inlineStr"/>
       <c r="P68" t="inlineStr">
         <is>
           <t>SpeechMap — which measures the performance of LLMs in complying with user prompts to generate disallowed, biased, or politically sensitive outputs — showed compliance scores for gpt-oss 120B hovering under 40%, near the bottom of peer open models, which indicates resistance to follow user requests and defaulting to guardrails, potentially at the expense of providing accurate information.</t>
@@ -11448,11 +11559,26 @@
           <t>BEFORE: A key rule of thumb we find useful here: If the reliability gain from a more expensive model or more inference time saves more of your or your users’ time (valued in terms of pay) than the model costs, going with the larger model is a good decision! || EVIDENCE: The rise of increasingly competitive open-weight LLMs, such as Meta’s Llama series, Mistral, DeepSeek, Gemma, Qwen, and now OpenAI’s GPT-OSS has added a critical dimension to the model selection landscape. || AFTER: Momentum behind this open ecosystem surged with the release of DeepSeek’s R1 reasoning model, competitive with OpenAI’s o1 but priced at roughly 30x lower API costs.</t>
         </is>
       </c>
-      <c r="T68" t="inlineStr"/>
-      <c r="U68" t="inlineStr"/>
-      <c r="V68" t="inlineStr"/>
-      <c r="W68" t="inlineStr"/>
-      <c r="X68" t="inlineStr"/>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
+      <c r="W68" t="inlineStr">
+        <is>
+          <t>entity_linking</t>
+        </is>
+      </c>
+      <c r="X68" t="inlineStr">
+        <is>
+          <t>The comparison concerns gpt-oss-120B and DeepSeek-R1. The tail is linked to the DeepSeek company rather than the competing model.</t>
+        </is>
+      </c>
       <c r="Y68" t="inlineStr">
         <is>
           <t>model:gpt_oss</t>
@@ -11516,9 +11642,6 @@
       <c r="AK68" t="n">
         <v>0.5214006304740906</v>
       </c>
-      <c r="AL68" t="inlineStr"/>
-      <c r="AM68" t="inlineStr"/>
-      <c r="AN68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -11583,7 +11706,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O69" t="inlineStr"/>
       <c r="P69" t="inlineStr">
         <is>
           <t>The OSI has faced calls to reconsider its decision about Faraone.</t>
@@ -11604,11 +11726,17 @@
           <t>BEFORE: LONDON — At a panel of leading open source AI experts at the third annual State of Open Con (SOOCon25), one thing quickly became clear: Even the pros are having trouble putting together the open source AI puzzle. || EVIDENCE: Moderator Alex Williams, The New Stack’s founder and publisher, opened the conversation by asking Sam Johnston, founder of the Open Source Alliance (OSA), to define the meaning of openness and AI, particularly concerning cost and reproducibility. || AFTER: “ At the heart of [ open source AI ] is reproducibility, ” said Johnston, whose group produced the Open Weight Definition (OWD).</t>
         </is>
       </c>
-      <c r="T69" t="inlineStr"/>
-      <c r="U69" t="inlineStr"/>
-      <c r="V69" t="inlineStr"/>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
       <c r="W69" t="inlineStr"/>
-      <c r="X69" t="inlineStr"/>
       <c r="Y69" t="inlineStr">
         <is>
           <t>org:open_source_alliance</t>
@@ -11672,9 +11800,6 @@
       <c r="AK69" t="n">
         <v>0.6949508786201477</v>
       </c>
-      <c r="AL69" t="inlineStr"/>
-      <c r="AM69" t="inlineStr"/>
-      <c r="AN69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -11739,7 +11864,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O70" t="inlineStr"/>
       <c r="P70" t="inlineStr">
         <is>
           <t>A two-person startup by the name of Nari Labs has introduced Dia, a 1.6 billion parameter text-to-speech (TTS) model designed to produce naturalistic dialogue directly from text prompts — and one of its creators claims it surpasses the performance of competing proprietary offerings from the likes of ElevenLabs, Google’s hit NotebookLM AI podcast generation product.</t>
@@ -11763,11 +11887,26 @@
 In standard dialogue scenarios, Dia handles both natural timing and nonverbal expressions better.</t>
         </is>
       </c>
-      <c r="T70" t="inlineStr"/>
-      <c r="U70" t="inlineStr"/>
-      <c r="V70" t="inlineStr"/>
-      <c r="W70" t="inlineStr"/>
-      <c r="X70" t="inlineStr"/>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
+      <c r="W70" t="inlineStr">
+        <is>
+          <t>schema_or_catalogue</t>
+        </is>
+      </c>
+      <c r="X70" t="inlineStr">
+        <is>
+          <t>The contexts support competition between Dia and ElevenLabs Studio. However, ElevenLabs Studio is a product/service, not a COMPANY as catalogued.</t>
+        </is>
+      </c>
       <c r="Y70" t="inlineStr">
         <is>
           <t>model:dia</t>
@@ -11831,9 +11970,6 @@
       <c r="AK70" t="n">
         <v>0.7012919187545776</v>
       </c>
-      <c r="AL70" t="inlineStr"/>
-      <c r="AM70" t="inlineStr"/>
-      <c r="AN70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -11898,7 +12034,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O71" t="inlineStr"/>
       <c r="P71" t="inlineStr">
         <is>
           <t>The Nemotron models also show how the company seems intent on becoming a one-stop shop for AI solutions.</t>
@@ -11924,10 +12059,17 @@
           <t>BEFORE: Enthusiasts will also be able to experience a range of NIM microservices using an upcoming release of the Nvidia ChatRTX tech demo. || EVIDENCE: To demonstrate how enthusiasts and developers can use NIM to build AI agents and assistants, Nvidia today previewed Project R2X, a vision-enabled PC avatar that can put information at a user’s fingertips, assist with desktop apps and video conference calls, read and summarize documents, and more. || AFTER: The avatar is rendered using Nvidia RTX Neural Faces, a new generative AI algorithm that augments traditional rasterization with entirely generated pixels.</t>
         </is>
       </c>
-      <c r="U71" t="inlineStr"/>
-      <c r="V71" t="inlineStr"/>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
       <c r="W71" t="inlineStr"/>
-      <c r="X71" t="inlineStr"/>
       <c r="Y71" t="inlineStr">
         <is>
           <t>model:nim</t>
@@ -12068,7 +12210,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O72" t="inlineStr"/>
       <c r="P72" t="inlineStr">
         <is>
           <t>DeepMind, the company he founded more than 10 years ago, which was acquired by Google in 2014, has been a key driving force behind Alphabet-owned Google's recent success with its AI products, including Gemini.</t>
@@ -12079,7 +12220,6 @@
           <t>In November, Google introduced Gemini 3, its latest model, which has been well-received by users and the market as the tech giant looked to allay fears it was falling behind rivals like OpenAI.</t>
         </is>
       </c>
-      <c r="R72" t="inlineStr"/>
       <c r="S72" t="inlineStr">
         <is>
           <t>BEFORE: We reimagined software development by moving beyond tools that assist coding to introducing powerful, agentic systems that collaborate with developers. || EVIDENCE: Key advances, such as the impressive coding capabilities in Gemini 3 and the launch of Google Antigravity, mark a new era in AI-assisted software development. || AFTER: This evolution was also clear across our core products, from AI-enabled features on the Pixel 10 and updates to AI Mode in Search, to AI-first innovations like the Gemini app and NotebookLM, which gained advanced features like Deep Research.
@@ -12091,10 +12231,17 @@
           <t>BEFORE: That pressure has only increased as competitors stepped up their game. || EVIDENCE: Google's Gemini 3, unveiled last month, has drawn solid reviews from users and analysts. || AFTER: OpenAI recently announced new updates to its GPT-5 AI model, while Anthropic debuted its Claude Opus 4.5 model in November shortly after releasing two other major models.</t>
         </is>
       </c>
-      <c r="U72" t="inlineStr"/>
-      <c r="V72" t="inlineStr"/>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
       <c r="W72" t="inlineStr"/>
-      <c r="X72" t="inlineStr"/>
       <c r="Y72" t="inlineStr">
         <is>
           <t>product:gemini_3</t>
@@ -12235,7 +12382,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O73" t="inlineStr"/>
       <c r="P73" t="inlineStr">
         <is>
           <t>The steps outlined on this page show you how to efficiently handle model inference on GPUs and customize models for diverse applications, equipping you with the tools to integrate advanced language models into your projects.</t>
@@ -12262,10 +12408,26 @@
           <t>BEFORE: It has also been developed in collaboration with industry experts. || EVIDENCE: Engineers from Google contributed to standardizing how LLM serving can plug into Kubernetes via new APIs, and Anyscale, the creators of Ray, have endorsed AIBrix’s approach to productionizing vLLM. || AFTER: This community momentum underscores that AIBrix isn’t an isolated tool.</t>
         </is>
       </c>
-      <c r="U73" t="inlineStr"/>
-      <c r="V73" t="inlineStr"/>
-      <c r="W73" t="inlineStr"/>
-      <c r="X73" t="inlineStr"/>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V73" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
+      <c r="W73" t="inlineStr">
+        <is>
+          <t>entity_boundary</t>
+        </is>
+      </c>
+      <c r="X73" t="inlineStr">
+        <is>
+          <t>The context concerns Google’s customized vLLM implementation. It does not establish that Google developed the original vLLM library.</t>
+        </is>
+      </c>
       <c r="Y73" t="inlineStr">
         <is>
           <t>technology:vllm</t>
@@ -12406,7 +12568,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O74" t="inlineStr"/>
       <c r="P74" t="inlineStr">
         <is>
           <t>Hold on.</t>
@@ -12432,10 +12593,17 @@
           <t>BEFORE: Skeptics worry it may divert resources from more effective and inclusive AI strategies, particularly as open-source models gain momentum. || EVIDENCE: The involvement of figures like Elon Musk, who occupies a unique position as both a government insider and a competitor to OpenAI through his xAI startup, adds further complexity to the discourse, as it challenges the project from within the same seat of power from which it was announced. || AFTER: The Stargate Project is undeniably one of the most ambitious undertakings in the history of artificial intelligence, but its ultimate impact remains uncertain.</t>
         </is>
       </c>
-      <c r="U74" t="inlineStr"/>
-      <c r="V74" t="inlineStr"/>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
       <c r="W74" t="inlineStr"/>
-      <c r="X74" t="inlineStr"/>
       <c r="Y74" t="inlineStr">
         <is>
           <t>org:openai</t>
@@ -12576,7 +12744,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O75" t="inlineStr"/>
       <c r="P75" t="inlineStr">
         <is>
           <t>One commenter highlighted the simplicity and utility of using Q-values for step scoring, while others speculated on future applications in geometric proofs and symbolic reasoning.</t>
@@ -12597,11 +12764,26 @@
           <t>BEFORE: Microsoft has introduced Phi-4, its latest lightweight and efficient language model, designed to rival larger AI systems like GPT-4 while maintaining a cost-effective and accessible framework. || EVIDENCE: Unlike closed-source models that demand significant computational power, Phi-4 is open-source and accessible on Hugging Face under an MIT license, thereby revolutionizing the landscape for AI developers globally. || AFTER: Optimized for Efficiency: Phi-4 performs remarkably well with fewer resources, making it ideal for smaller businesses and researchers.</t>
         </is>
       </c>
-      <c r="T75" t="inlineStr"/>
-      <c r="U75" t="inlineStr"/>
-      <c r="V75" t="inlineStr"/>
-      <c r="W75" t="inlineStr"/>
-      <c r="X75" t="inlineStr"/>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V75" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
+      <c r="W75" t="inlineStr">
+        <is>
+          <t>entity_boundary</t>
+        </is>
+      </c>
+      <c r="X75" t="inlineStr">
+        <is>
+          <t>Both the primary and supporting evidence assign the MIT license specifically to Phi-4, not the entire Phi model family.</t>
+        </is>
+      </c>
       <c r="Y75" t="inlineStr">
         <is>
           <t>model:phi</t>
@@ -12665,9 +12847,6 @@
       <c r="AK75" t="n">
         <v>0.6006895303726196</v>
       </c>
-      <c r="AL75" t="inlineStr"/>
-      <c r="AM75" t="inlineStr"/>
-      <c r="AN75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -12732,7 +12911,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O76" t="inlineStr"/>
       <c r="P76" t="inlineStr">
         <is>
           <t>But processors remain a sticking point.</t>
@@ -12753,11 +12931,26 @@
           <t>BEFORE: How it works: The Chinese government’s resistance to AI processors from U.S. vendors signals rising confidence in the nation’s AI capabilities, as the U.S. seeks to return to selling advanced processors in China after blocking such sales in recent months. || EVIDENCE: China is helping the domestic semiconductor industry to compete against U.S. designers like Nvidia and AMD and the Taiwanese manufacturer TSMC, which fabricates their products, by providing funds and tax incentives and applying pressure to Chinese AI companies to buy processors made domestically. || AFTER: Meanwhile, Chinese vendors aim to close the performance gap between their products and those of U.S. competitors.</t>
         </is>
       </c>
-      <c r="T76" t="inlineStr"/>
-      <c r="U76" t="inlineStr"/>
-      <c r="V76" t="inlineStr"/>
-      <c r="W76" t="inlineStr"/>
-      <c r="X76" t="inlineStr"/>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V76" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
+      <c r="W76" t="inlineStr">
+        <is>
+          <t>entity_linking</t>
+        </is>
+      </c>
+      <c r="X76" t="inlineStr">
+        <is>
+          <t>China’s semiconductor industry competes with NVIDIA and TSMC. Neither context establishes competition between NVIDIA and TSMC; support 2 says TSMC fabricates their products.</t>
+        </is>
+      </c>
       <c r="Y76" t="inlineStr">
         <is>
           <t>org:nvidia</t>
@@ -12821,9 +13014,6 @@
       <c r="AK76" t="n">
         <v>0.6900020241737366</v>
       </c>
-      <c r="AL76" t="inlineStr"/>
-      <c r="AM76" t="inlineStr"/>
-      <c r="AN76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -12888,7 +13078,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O77" t="inlineStr"/>
       <c r="P77" t="inlineStr">
         <is>
           <t>26.</t>
@@ -12909,11 +13098,17 @@
           <t>BEFORE: The forecasts are available on Flood Hub along with our riverine flood forecasts, which now cover 2B people in 150 countries for the most significant flood events. || EVIDENCE: WeatherNext and flood forecasting models are part of Google Earth AI, a collection of geospatial models and datasets, designed to transform planetary information into actionable intelligence. || AFTER: It is already helping enterprises, cities and nonprofits with challenges from environmental monitoring and disaster response to supporting public health.</t>
         </is>
       </c>
-      <c r="T77" t="inlineStr"/>
-      <c r="U77" t="inlineStr"/>
-      <c r="V77" t="inlineStr"/>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V77" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
       <c r="W77" t="inlineStr"/>
-      <c r="X77" t="inlineStr"/>
       <c r="Y77" t="inlineStr">
         <is>
           <t>model:weathernext</t>
@@ -12977,9 +13172,6 @@
       <c r="AK77" t="n">
         <v>0.6889326572418213</v>
       </c>
-      <c r="AL77" t="inlineStr"/>
-      <c r="AM77" t="inlineStr"/>
-      <c r="AN77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -13044,7 +13236,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O78" t="inlineStr"/>
       <c r="P78" t="inlineStr">
         <is>
           <t>LTX 2.3, Lightricks’ state-of-the-art audio-video model, released earlier this month, now has support for NVFP4 and FP8 distilled models, accelerating performance by 2.1x.</t>
@@ -13065,11 +13256,17 @@
           <t>BEFORE: Learn more about the latest on NVIDIA open models. || EVIDENCE: LTX 2.3, Lightricks’ state-of-the-art audio-video model, released earlier this month, now has support for NVFP4 and FP8 distilled models, accelerating performance by 2.1x. || AFTER: Learn more about Lightricks’ LTX 2.3 model.</t>
         </is>
       </c>
-      <c r="T78" t="inlineStr"/>
-      <c r="U78" t="inlineStr"/>
-      <c r="V78" t="inlineStr"/>
+      <c r="U78" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V78" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
       <c r="W78" t="inlineStr"/>
-      <c r="X78" t="inlineStr"/>
       <c r="Y78" t="inlineStr">
         <is>
           <t>product:ltx_2_3</t>
@@ -13133,9 +13330,6 @@
       <c r="AK78" t="n">
         <v>0.7678853273391724</v>
       </c>
-      <c r="AL78" t="inlineStr"/>
-      <c r="AM78" t="inlineStr"/>
-      <c r="AN78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -13200,7 +13394,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O79" t="inlineStr"/>
       <c r="P79" t="inlineStr">
         <is>
           <t>Huang said the company plans to release a rack-scale architecture for AI data centers that will connect 576 next-generation GPUs in the second half of 2027.</t>
@@ -13226,10 +13419,26 @@
           <t>BEFORE: But the clearest signal to date came this week. || EVIDENCE: At Nvidia's annual developer conference, GTC, Huang launched NemoClaw, an open-source, chip-agnostic platform for building and deploying AI agents – autonomous software programs at the center of the latest advancements in the industry. || AFTER: "Every company in the world should have an agentic system strategy," Huang said.</t>
         </is>
       </c>
-      <c r="U79" t="inlineStr"/>
-      <c r="V79" t="inlineStr"/>
-      <c r="W79" t="inlineStr"/>
-      <c r="X79" t="inlineStr"/>
+      <c r="U79" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V79" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
+      <c r="W79" t="inlineStr">
+        <is>
+          <t>wrong_predicate</t>
+        </is>
+      </c>
+      <c r="X79" t="inlineStr">
+        <is>
+          <t>GTC is the conference at which Huang announced technologies and a roadmap. The contexts do not say that he announced GTC itself. GTC is also incorrectly typed as BENCHMARK.</t>
+        </is>
+      </c>
       <c r="Y79" t="inlineStr">
         <is>
           <t>benchmark:gtc</t>
@@ -13370,7 +13579,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O80" t="inlineStr"/>
       <c r="P80" t="inlineStr">
         <is>
           <t>We have validated the model's performance on context lengths of up to 131,072 tokens using the YaRN method.</t>
@@ -13395,11 +13603,26 @@
 All the notable open-source frameworks implement static YaRN, which means the scaling factor remains constant regardless of input length, potentially impacting performance on shorter texts.</t>
         </is>
       </c>
-      <c r="T80" t="inlineStr"/>
-      <c r="U80" t="inlineStr"/>
-      <c r="V80" t="inlineStr"/>
-      <c r="W80" t="inlineStr"/>
-      <c r="X80" t="inlineStr"/>
+      <c r="U80" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V80" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
+      <c r="W80" t="inlineStr">
+        <is>
+          <t>entity_linking</t>
+        </is>
+      </c>
+      <c r="X80" t="inlineStr">
+        <is>
+          <t>YaRN is supported by Transformers and vLLM. The sentence does not state that Transformers is supported by vLLM.</t>
+        </is>
+      </c>
       <c r="Y80" t="inlineStr">
         <is>
           <t>product:transformers</t>
@@ -13463,9 +13686,6 @@
       <c r="AK80" t="n">
         <v>0.6058963537216187</v>
       </c>
-      <c r="AL80" t="inlineStr"/>
-      <c r="AM80" t="inlineStr"/>
-      <c r="AN80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -13530,7 +13750,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O81" t="inlineStr"/>
       <c r="P81" t="inlineStr">
         <is>
           <t>Nvidia will resume sales of H20 processors in China.</t>
@@ -13552,11 +13771,17 @@
 “</t>
         </is>
       </c>
-      <c r="T81" t="inlineStr"/>
-      <c r="U81" t="inlineStr"/>
-      <c r="V81" t="inlineStr"/>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V81" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
       <c r="W81" t="inlineStr"/>
-      <c r="X81" t="inlineStr"/>
       <c r="Y81" t="inlineStr">
         <is>
           <t>product:h20</t>
@@ -13620,9 +13845,6 @@
       <c r="AK81" t="n">
         <v>0.5332844853401184</v>
       </c>
-      <c r="AL81" t="inlineStr"/>
-      <c r="AM81" t="inlineStr"/>
-      <c r="AN81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -13719,10 +13941,17 @@
 Stability AI, founded in 2019 and headquartered in London, UK, has played a pivotal role in bringing generative AI to public attention through its Stable Diffusion image generation model. || AFTER: The company has expanded its AI capabilities beyond images to include video, audio, and 3D media generation, positioning itself as a leader in enterprise-grade creative AI solutions.</t>
         </is>
       </c>
-      <c r="U82" t="inlineStr"/>
-      <c r="V82" t="inlineStr"/>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V82" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
       <c r="W82" t="inlineStr"/>
-      <c r="X82" t="inlineStr"/>
       <c r="Y82" t="inlineStr">
         <is>
           <t>org:stability_ai</t>
@@ -13863,7 +14092,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O83" t="inlineStr"/>
       <c r="P83" t="inlineStr">
         <is>
           <t>The road map reflects the one-year release cadence Nvidia put into action for its data center GPUs and associated platforms last year with the launch of its H200 GPU, which was followed with the Blackwell-based platforms that started shipping a few months ago.</t>
@@ -13884,11 +14112,17 @@
           <t>BEFORE: Nvidia has yet to confirm any plans for a system-on-chip for Windows PCs. || EVIDENCE: Nvidia in March revealed plans to release new Spectrum-X Ethernet and Quantum-X InfiniBand networking switches that use silicon photonics to lower energy consumption and, as a result, enable larger-scale GPU clusters. || AFTER: At its GTC 2025 event, the company said the Quantum-X Photonics InfiniBand switches will launch later this year while the Spectrum-X Photonics Ethernet switches will arrive next year from “ leading infrastructure and system vendors.</t>
         </is>
       </c>
-      <c r="T83" t="inlineStr"/>
-      <c r="U83" t="inlineStr"/>
-      <c r="V83" t="inlineStr"/>
+      <c r="U83" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V83" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
       <c r="W83" t="inlineStr"/>
-      <c r="X83" t="inlineStr"/>
       <c r="Y83" t="inlineStr">
         <is>
           <t>product:spectrum_x_ethernet</t>
@@ -13952,9 +14186,6 @@
       <c r="AK83" t="n">
         <v>0.6007272601127625</v>
       </c>
-      <c r="AL83" t="inlineStr"/>
-      <c r="AM83" t="inlineStr"/>
-      <c r="AN83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -14019,7 +14250,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O84" t="inlineStr"/>
       <c r="P84" t="inlineStr">
         <is>
           <t>Google's data centres used 20 per cent more water in 2022 than in 2021.</t>
@@ -14040,11 +14270,26 @@
           <t>BEFORE: Shaolei Ren, an associate professor at the University of California, Riverside who has studied the water costs of computation for the past decade, has worked to make this hidden impact visible. || EVIDENCE: His research reveals that training GPT-3 in Microsoft's state-of-the-art U.S. data centres directly evaporated approximately 700,000 litres of clean freshwater. || AFTER: The training of GPT-4 at similar facilities consumed an estimated total of 5.4 million litres of water.</t>
         </is>
       </c>
-      <c r="T84" t="inlineStr"/>
-      <c r="U84" t="inlineStr"/>
-      <c r="V84" t="inlineStr"/>
-      <c r="W84" t="inlineStr"/>
-      <c r="X84" t="inlineStr"/>
+      <c r="U84" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V84" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
+      <c r="W84" t="inlineStr">
+        <is>
+          <t>wrong_predicate</t>
+        </is>
+      </c>
+      <c r="X84" t="inlineStr">
+        <is>
+          <t>The primary evidence concerns Microsoft hosting GPT-3. Support 2 concerns training in Microsoft data centres, not Microsoft developing the model.</t>
+        </is>
+      </c>
       <c r="Y84" t="inlineStr">
         <is>
           <t>model:gpt_3_2</t>
@@ -14108,9 +14353,6 @@
       <c r="AK84" t="n">
         <v>0.5717583894729614</v>
       </c>
-      <c r="AL84" t="inlineStr"/>
-      <c r="AM84" t="inlineStr"/>
-      <c r="AN84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -14175,7 +14417,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O85" t="inlineStr"/>
       <c r="P85" t="inlineStr">
         <is>
           <t>As with GPT-4o, the models’ responses included both the system prompt and the injected function definitions, but unlike GPT-4o, both models attempted to call our fake function.;;
@@ -14197,11 +14438,26 @@
           <t>BEFORE: One of Kimi K2's strengths is in writing computer code for applications, an area in which businesses see potential to reduce or replace staff with generative AI. || EVIDENCE: OpenAI's U.S. rival Anthropic focused on coding with its Claude Opus 4 model released in late May. || AFTER: In its release announcement on social media platforms X and GitHub, Moonshot claimed Kimi K2 surpassed Claude Opus 4 on two benchmarks, and had better overall performance than OpenAI's coding-focused GPT-4.1 model, based on several industry metrics.</t>
         </is>
       </c>
-      <c r="T85" t="inlineStr"/>
-      <c r="U85" t="inlineStr"/>
-      <c r="V85" t="inlineStr"/>
-      <c r="W85" t="inlineStr"/>
-      <c r="X85" t="inlineStr"/>
+      <c r="U85" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V85" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
+      <c r="W85" t="inlineStr">
+        <is>
+          <t>entity_linking</t>
+        </is>
+      </c>
+      <c r="X85" t="inlineStr">
+        <is>
+          <t>OpenAI’s ownership applies to GPT-4o and o4-mini in the list. Support 2 explicitly identifies Claude Opus 4 as Anthropic’s model.</t>
+        </is>
+      </c>
       <c r="Y85" t="inlineStr">
         <is>
           <t>product:claude_opus_4</t>
@@ -14265,9 +14521,6 @@
       <c r="AK85" t="n">
         <v>0.5506665110588074</v>
       </c>
-      <c r="AL85" t="inlineStr"/>
-      <c r="AM85" t="inlineStr"/>
-      <c r="AN85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -14332,7 +14585,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O86" t="inlineStr"/>
       <c r="P86" t="inlineStr">
         <is>
           <t>The threat actor used a common vector — data files using the Pickle format — with a new technique, dubbed "NullifAI," to evade detection.</t>
@@ -14353,11 +14605,17 @@
           <t>BEFORE: Other models — such as OpenAI's o3-mini model, which boasts more stringent alignment — has already been jail broken by researchers. || EVIDENCE: These problems are unique to AI systems and the boundaries of how to test for such weaknesses remains a fertile field for researchers, says ReversingLabs ' Pericin. || AFTER: "There is already research about what kind of prompts would trigger the model to behave in an unpredictable way, divulge confidential information, or teach things that could be harmful," he says.</t>
         </is>
       </c>
-      <c r="T86" t="inlineStr"/>
-      <c r="U86" t="inlineStr"/>
-      <c r="V86" t="inlineStr"/>
+      <c r="U86" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V86" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
       <c r="W86" t="inlineStr"/>
-      <c r="X86" t="inlineStr"/>
       <c r="Y86" t="inlineStr">
         <is>
           <t>person:tomislav_pericin</t>
@@ -14421,9 +14679,6 @@
       <c r="AK86" t="n">
         <v>0.5312821269035339</v>
       </c>
-      <c r="AL86" t="inlineStr"/>
-      <c r="AM86" t="inlineStr"/>
-      <c r="AN86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -14488,7 +14743,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O87" t="inlineStr"/>
       <c r="P87" t="inlineStr">
         <is>
           <t>As a regular user of voice transcription services, I can say firsthand that speech recognition AI is not perfect, but it is improving.</t>
@@ -14509,11 +14763,26 @@
           <t>BEFORE: Mistral stated that Voxtral outperformed existing voice models, including OpenAI’s Whisper, Gemini 2.5 Flash and Scribe from ElevenLabs. || EVIDENCE: Voxtral presented fewer word errors compared to Whisper, which is currently considered the best automatic speech recognition model available. || AFTER: In terms of audio understanding, Voxtral Small is “ competitive with GPT-4o-mini and Gemini 2.5 Flash across all tasks, achieving state-of-the-art performance in Speech Translation.</t>
         </is>
       </c>
-      <c r="T87" t="inlineStr"/>
-      <c r="U87" t="inlineStr"/>
-      <c r="V87" t="inlineStr"/>
-      <c r="W87" t="inlineStr"/>
-      <c r="X87" t="inlineStr"/>
+      <c r="U87" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V87" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
+      <c r="W87" t="inlineStr">
+        <is>
+          <t>entity_linking</t>
+        </is>
+      </c>
+      <c r="X87" t="inlineStr">
+        <is>
+          <t>Voxtral is the model reported to outperform Whisper. Mistral is the company making the claim, not the compared model.</t>
+        </is>
+      </c>
       <c r="Y87" t="inlineStr">
         <is>
           <t>model:mistral</t>
@@ -14577,9 +14846,6 @@
       <c r="AK87" t="n">
         <v>0.5371658205986023</v>
       </c>
-      <c r="AL87" t="inlineStr"/>
-      <c r="AM87" t="inlineStr"/>
-      <c r="AN87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -14644,7 +14910,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O88" t="inlineStr"/>
       <c r="P88" t="inlineStr">
         <is>
           <t>NVIDIA Agent Toolkit and NVIDIA NemoClaw blueprints give developers an open source platform to build production agents on Foundry.</t>
@@ -14668,11 +14933,17 @@
 Accelerated computing begins with NVIDIA CUDA‑X libraries across the stack — from cuDNN and TensorRT‑LLM for deep learning, to RAPIDS (cuDF/cuML) for data science, cuOpt for decision optimization, cuLitho for computational lithograph, CUDA‑Q and cuQuantum for quantum and hybrid quantum‑classical computing, and more. || AFTER: “ This really is the treasure of our company, ” Huang said, before teeing up a video showing what CUDA-X can do.</t>
         </is>
       </c>
-      <c r="T88" t="inlineStr"/>
-      <c r="U88" t="inlineStr"/>
-      <c r="V88" t="inlineStr"/>
+      <c r="U88" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V88" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
       <c r="W88" t="inlineStr"/>
-      <c r="X88" t="inlineStr"/>
       <c r="Y88" t="inlineStr">
         <is>
           <t>technology:cuopt</t>
@@ -14736,9 +15007,6 @@
       <c r="AK88" t="n">
         <v>0.6996411681175232</v>
       </c>
-      <c r="AL88" t="inlineStr"/>
-      <c r="AM88" t="inlineStr"/>
-      <c r="AN88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -14803,7 +15071,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O89" t="inlineStr"/>
       <c r="P89" t="inlineStr">
         <is>
           <t>A two-person startup by the name of Nari Labs has introduced Dia, a 1.6 billion parameter text-to-speech (TTS) model designed to produce naturalistic dialogue directly from text prompts — and one of its creators claims it surpasses the performance of competing proprietary offerings from the likes of ElevenLabs, Google’s hit NotebookLM AI podcast generation product.</t>
@@ -14827,11 +15094,26 @@
 In standard dialogue scenarios, Dia handles both natural timing and nonverbal expressions better.</t>
         </is>
       </c>
-      <c r="T89" t="inlineStr"/>
-      <c r="U89" t="inlineStr"/>
-      <c r="V89" t="inlineStr"/>
-      <c r="W89" t="inlineStr"/>
-      <c r="X89" t="inlineStr"/>
+      <c r="U89" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V89" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
+      <c r="W89" t="inlineStr">
+        <is>
+          <t>entity_linking</t>
+        </is>
+      </c>
+      <c r="X89" t="inlineStr">
+        <is>
+          <t>The competing model is Dia, created by Nari Labs. Nari is incorrectly linked as an AI_MODEL. ElevenLabs Studio is also incorrectly typed as COMPANY.</t>
+        </is>
+      </c>
       <c r="Y89" t="inlineStr">
         <is>
           <t>model:nari</t>
@@ -14895,9 +15177,6 @@
       <c r="AK89" t="n">
         <v>0.7167259454727173</v>
       </c>
-      <c r="AL89" t="inlineStr"/>
-      <c r="AM89" t="inlineStr"/>
-      <c r="AN89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -14962,7 +15241,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O90" t="inlineStr"/>
       <c r="P90" t="inlineStr">
         <is>
           <t>A key rule of thumb we find useful here: If the reliability gain from a more expensive model or more inference time saves more of your or your users’ time (valued in terms of pay) than the model costs, going with the larger model is a good decision!</t>
@@ -14988,10 +15266,26 @@
           <t>BEFORE: Together, these teams will work toward the realization of superintelligence — AI that exceeds human intelligence in all aspects. || EVIDENCE: The move comes on the heels of a disappointing showing from Meta’s Llama 4 models, which left the company trailing behind rivals like OpenAI, Anthropic, Google and DeepSeek. || AFTER: To close the gap, Zuckerberg has gone on an aggressive hiring spree, offering signing bonuses of up to $ 1 billion to lure some of the industry’s top players over to MSL.</t>
         </is>
       </c>
-      <c r="U90" t="inlineStr"/>
-      <c r="V90" t="inlineStr"/>
-      <c r="W90" t="inlineStr"/>
-      <c r="X90" t="inlineStr"/>
+      <c r="U90" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="V90" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
+      <c r="W90" t="inlineStr">
+        <is>
+          <t>entity_linking</t>
+        </is>
+      </c>
+      <c r="X90" t="inlineStr">
+        <is>
+          <t>The contexts compare model offerings and describe Meta competing with OpenAI. The extracted relation instead links the Llama model family directly to the OpenAI company.</t>
+        </is>
+      </c>
       <c r="Y90" t="inlineStr">
         <is>
           <t>model:llama</t>
@@ -15132,7 +15426,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O91" t="inlineStr"/>
       <c r="P91" t="inlineStr">
         <is>
           <t>A statement from Windsurf said: “ With this acquisition, two world-class teams are joining forces to shape the next era of AI coding — and we’re just getting started. ”</t>
@@ -15153,11 +15446,17 @@
           <t>BEFORE: To zoom out just a little, AI coding tools have exploded these past couple of years, morphing from smart autocomplete widgets into full-blown assistants that promise everything from bug fixes to multi-file refactors. || EVIDENCE: The landscape is dominated by a handful of heavyweights: GitHub Copilot, the default for many developers; Cursor, a VC-fuelled juggernaut pushing a tightly integrated, closed-stack model; Claude Code, Anthropic’s terminal-first agent built around deep codebase awareness; and newcomers like Windsurf (recently acquired by Cognition) and Replit, each promising deeper hooks into proprietary models. || AFTER: Most of these platforms fall into two broad camps: the closed, single-model assistants tied tightly to one provider, and the convenience-first tools that wrap proprietary models in polished interfaces with an implicit degree of lock-in.</t>
         </is>
       </c>
-      <c r="T91" t="inlineStr"/>
-      <c r="U91" t="inlineStr"/>
-      <c r="V91" t="inlineStr"/>
+      <c r="U91" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V91" t="inlineStr">
+        <is>
+          <t>jihyeon choung</t>
+        </is>
+      </c>
       <c r="W91" t="inlineStr"/>
-      <c r="X91" t="inlineStr"/>
       <c r="Y91" t="inlineStr">
         <is>
           <t>org:windsurf</t>
@@ -15221,9 +15520,6 @@
       <c r="AK91" t="n">
         <v>0.8202033042907715</v>
       </c>
-      <c r="AL91" t="inlineStr"/>
-      <c r="AM91" t="inlineStr"/>
-      <c r="AN91" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>

<commit_message>
feat(wp3): apply the final human review to the Korean knowledge graph notebook
</commit_message>
<xml_diff>
--- a/artifacts/stage1_wp3/evaluation/relation_correction/relation_review_corrected_seed2026.xlsx
+++ b/artifacts/stage1_wp3/evaluation/relation_correction/relation_review_corrected_seed2026.xlsx
@@ -714,6 +714,24 @@
           <t>BEFORE: According to independent testing from Artificial Analysis and Arena.ai, Kimi K3’s capabilities are competitive with both Anthropic’s Fable 5, which was released last month, and OpenAI’s GPT-5.6, which was released just a week prior. || EVIDENCE: Back in February, though, Anthropic accused three Chinese AI companies âMoonshot, DeepSeek, and Minimaxâ of violating Anthropic’s terms of service and regional access restrictions to “ illicitly ” extract the capabilities of its Claude model and use that to improve their own. || AFTER: Around the same time, OpenAI sent a memo to the House of Representatives, accusing DeepSeek of a similar tactic, claiming that it is trying to “ free-ride on the capabilities developed by OpenAI and other U.S. frontier labs. ”</t>
         </is>
       </c>
+      <c r="U2" t="b">
+        <v>0</v>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>entity_linking</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>DeepSeek and Moonshot are accused of distillation by Anthropic. Support 2 lists them as competitors of Ant's Ling-1T, not of each other</t>
+        </is>
+      </c>
       <c r="Y2" t="inlineStr">
         <is>
           <t>org:deepseek</t>
@@ -881,6 +899,14 @@
           <t>BEFORE: Open-source AI is accelerating innovation across industries, and NVIDIA DGX Spark and DGX Station are built to help developers turn innovation into impact. || EVIDENCE: NVIDIA today unveiled at the CES trade show how the DGX Spark and DGX Station deskside AI supercomputers let developers harness the latest open and frontier AI models on a local deskside system, from 100-billion-parameter models on DGX Spark to 1-trillion-parameter models on DGX Station. || AFTER: Powered by the NVIDIA Grace Blackwell architecture, with large unified memory and petaflop-level AI performance, these systems give developers new capabilities to develop locally and easily scale to the cloud.</t>
         </is>
       </c>
+      <c r="U3" t="b">
+        <v>1</v>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
       <c r="Y3" t="inlineStr">
         <is>
           <t>hardware:dgx_spark</t>
@@ -1047,6 +1073,14 @@
           <t>BEFORE: It comes ahead of the kickoff of Llamacon 2025, Meta’s first AI developer conference taking place this week at its office campus headquarters in Palo Alto, California, centered around its Llama model family and general AI developer tools and advances. || EVIDENCE: With the rise of more AI model challengers in the open source and proprietary domains — including everyone from OpenAI with ChatGPT to Google with its Gemini 2.5 model family and lesser-known (at least, to Western audiences) brands like Alibaba’s new Qwen 3 — Meta is keen to show off the power and capabilities of its own, in-house Llama 4 models. || AFTER: It is also seeking to make the case to third-party software developers that Llama 4 is a powerful and flexible open (ish) source model family they can trust to build their enterprise products atop of.</t>
         </is>
       </c>
+      <c r="U4" t="b">
+        <v>1</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
       <c r="Y4" t="inlineStr">
         <is>
           <t>org:meta</t>
@@ -1205,6 +1239,24 @@
 Nari Labs, a two-person startup, released Dia, a 1.6 billion parameter text-to-speech model that generates naturalistic dialogue directly from text prompts. || EVIDENCE: The model supports advanced features like emotional tone, speaker tagging, and nonverbal audio cues such as laughs and coughs — capabilities that co-creator Toby Kim claims surpass competing offerings from ElevenLabs and Google’s NotebookLM. || AFTER: Side-by-side comparisons show Dia handling natural timing, nonverbal expressions, and emotional range quite effectively, with examples demonstrating how it properly interprets cues that other models simply read aloud or skip entirely.</t>
         </is>
       </c>
+      <c r="U5" t="b">
+        <v>0</v>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>entity_linking</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>ElevenLabs and Google are both competitors of Nari Labs' Dia, not of each other</t>
+        </is>
+      </c>
       <c r="Y5" t="inlineStr">
         <is>
           <t>org:elevenlabs</t>
@@ -1357,6 +1409,14 @@
           <t>BEFORE: Hold on. || EVIDENCE: Interestingly, the source code for both the V3 and R1 models and their V2 predecessor are all available on GitHub, which is more than you can say for the proprietary models from OpenAI, Google, Anthropic, xAI, and others. || AFTER: But what we want to know – and what is roiling the tech titans today – is precisely how DeepSeek was able to take a few thousand crippled “ Hopper ” H800 GPU accelerators from Nvidia, which have some of their performance capped, and create an MoE foundation model that can stand toe-to-toe with the best that OpenAI, Google, and Anthropic can do with their largest models as they are trained on tens of thousands of uncrimped GPU accelerators.</t>
         </is>
       </c>
+      <c r="U6" t="b">
+        <v>1</v>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
       <c r="Y6" t="inlineStr">
         <is>
           <t>org:google</t>
@@ -1518,6 +1578,14 @@
 Agent Trainer aims to boost business performance and customer satisfaction by delivering ROI through lower training costs, tailored training recommendations and faster agent proficiency—ultimately reducing turnover, Google said. || AFTER: Targeting the Contact Center-as-a-Service (CCaaS) market, Google Cloud has created a new stand-alone agent desktop application.</t>
         </is>
       </c>
+      <c r="U7" t="b">
+        <v>1</v>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
       <c r="Y7" t="inlineStr">
         <is>
           <t>person:antony_passemard</t>
@@ -1670,6 +1738,14 @@
           <t>BEFORE: More than $ 700 billion was wiped from the value of the world’s largest technology companies on Monday after the emergence of a cut-price Chinese rival to ChatGPT raised doubts over whether America can sustain its lead in artificial intelligence. || EVIDENCE: California-based Nvidia, whose share price has been turbocharged by speculation that generative AI would fuel rapid growth in demand for its computer chips, lost $ 590 billion, and its crown as the world’s most valuable public company. || AFTER: DeepSeek said it has produced a free open-source assistant that uses lower-cost chips and less data than its American rivals.</t>
         </is>
       </c>
+      <c r="U8" t="b">
+        <v>1</v>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
       <c r="Y8" t="inlineStr">
         <is>
           <t>org:nvidia</t>
@@ -1831,6 +1907,24 @@
 Bun’s frontend dev server is going to get “ automatic workspaces ” support in Chrome DevTools, which means developers can edit the files in the browser. || AFTER: Bun is a JavaScript runtime designed as a drop-in replacement for Node.js.</t>
         </is>
       </c>
+      <c r="U9" t="b">
+        <v>0</v>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>reversed_direction</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>Chrome DevTools supports Bun's dev server, not the reverse</t>
+        </is>
+      </c>
       <c r="Y9" t="inlineStr">
         <is>
           <t>product:chrome_devtools</t>
@@ -1978,6 +2072,24 @@
           <t>EVIDENCE: BEIJING — DeepSeek's artificial intelligence breakthrough is stirring up China's venture capital world after three straight years of decline. || AFTER: As DeepSeek released its OpenAI rival in late January, AI drug discovery company Insilico Medicine was finalizing a $ 110 million series E financing round led by Hong Kong-based Value Partners, the startup's CEO and founder Alex Zhavoronkov told CNBC in an exclusive interview.</t>
         </is>
       </c>
+      <c r="U10" t="b">
+        <v>0</v>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>insufficient_context</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>Beijing refers to the government. HQ not stated</t>
+        </is>
+      </c>
       <c r="Y10" t="inlineStr">
         <is>
           <t>org:deepseek</t>
@@ -2125,6 +2237,24 @@
           <t>BEFORE: But those tools aren't officially available in China. || EVIDENCE: Beijing's firewall keeps out Google and Facebook and their AI models, and Anthropic cited national security concerns in its ban on China-owned entities from using Claude, widely considered the best AI for coding right now. || AFTER: Yet discussion of leading U.S. models is prevalent enough on Chinese social media to signal that such technologies are being used by local developers.</t>
         </is>
       </c>
+      <c r="U11" t="b">
+        <v>0</v>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>entity_linking</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>the competitor is Meta ('the Facebook parent')</t>
+        </is>
+      </c>
       <c r="Y11" t="inlineStr">
         <is>
           <t>org:facebook</t>
@@ -2286,6 +2416,14 @@
           <t>BEFORE: He draws inspiration from nature and his surroundings, and attempts to capture elements of human life and the current world that we live in. || EVIDENCE: More about Polygreen Culture and Art Initiative (PCAI) and “ pi ” PCAI is a cultural organization founded by Athanasios Polychronopoulos, Polygreen CEO, as a means to increase environmental awareness through an annual programme of commissions, contemporary art exhibitions, artist residencies, workshops, conferences and sponsorships. || AFTER: The PCAI Art Collection focuses on commissions and acquisitions of moving image and contemporary art while providing artists with the means and resources to create an artwork inspired by urgent environmental, sociological and philosophical issues, allowing for their absolute freedom of expression and critical inquiry.</t>
         </is>
       </c>
+      <c r="U12" t="b">
+        <v>1</v>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
       <c r="Y12" t="inlineStr">
         <is>
           <t>org:pcai</t>
@@ -2440,6 +2578,24 @@
 While those other players do offer developer tools and products, the continual evolution of OpenAI’s developer platform makes it a hard proposition to beat as a “ one stop shop ” for those looking to leverage the latest AI advances in a clean, easy-to-use, fast and affordable way. || EVIDENCE: In a move certain to send the AI blogosphere and social media space aflutter, OpenAI is getting back into open source in a big way with the release of its Agents SDK, a toolkit designed to help developers manage, coordinate and optimize agent workflows — even building agents powered by other, non-OpenAI models such as those by competitors Anthropic and Google, or open-source models from DeepSeek, Qwen, Mistral and Meta’s Llama family. || AFTER: “ The Agent SDK is open-source, allowing enterprises to mix and match different models, ” said Godement.</t>
         </is>
       </c>
+      <c r="U13" t="b">
+        <v>0</v>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>entity_linking</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>DeepSeek, Mistral and Llama are listed as open competitors of OpenAI's model, not of each other</t>
+        </is>
+      </c>
       <c r="Y13" t="inlineStr">
         <is>
           <t>model:llama</t>
@@ -2605,6 +2761,14 @@
           <t>BEFORE: However, this isn’t unique to AMD. || EVIDENCE: In MLPerf training, Nvidia has previously demonstrated a 1.3X improvement of performance over its initial “ Hopper ” H100 submissions thanks in part to software optimizations. || AFTER: With that said, driving these kinds of software optimizations are arguably even more important for AMD, which trails its rival in both market share and awareness.</t>
         </is>
       </c>
+      <c r="U14" t="b">
+        <v>1</v>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
       <c r="Y14" t="inlineStr">
         <is>
           <t>platform:hopper</t>
@@ -2771,6 +2935,14 @@
 Determining which search strategy is best is still an active area of research, but there are a lot of great resources on HuggingFace which provide examples for how these search strategies can be implemented for your use case. || EVIDENCE: OpenAI’s o1 model announced in September 2024 was one of the first models designed to "think" before responding to users. || AFTER: Although it takes longer to get a response from o1 compared to models like GPT-4o, o1’s responses are typically better for more advanced tasks since it generates chain of thought sequences that help it break down and solve problems.</t>
         </is>
       </c>
+      <c r="U15" t="b">
+        <v>1</v>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
       <c r="Y15" t="inlineStr">
         <is>
           <t>model:o1_model</t>
@@ -2931,6 +3103,14 @@
           <t>BEFORE: Far from being a “ powerful chip ” as some have claimed, the H20 actually has worse computational performance and energy efficiency than Nvidia’s older A100 chips, launched back in 2020. || EVIDENCE: Moreover, Huawei has been able to improve the computational performance of its Ascend chips, even after switching production from Taiwanese chip manufacturer TSMC to China’s own SMIC following U.S. export controls. || AFTER: Perhaps more importantly, Huawei has been making significant progress at the level of AI computing systems.</t>
         </is>
       </c>
+      <c r="U16" t="b">
+        <v>1</v>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
       <c r="Y16" t="inlineStr">
         <is>
           <t>hardware:ascend_chips</t>
@@ -3085,6 +3265,24 @@
           <t>BEFORE: “ DeepSeek is definitely reshaping the AI landscape, challenging giants with open-source ambition and state-of-the-art innovations, ” says Kaoutar El Maghraoui, a Principal Research Scientist and Manager at IBM AI Hardware. || EVIDENCE: Meanwhile, ByteDance, the Chinese tech giant that owns TikTok, recently announced its own reasoning agent, UI-TARS, which it claims outperforms OpenAI’s GPT-4o, Anthropic’s Claude and Google’s Gemini on certain benchmarks. || AFTER: ByteDance’s agent can read graphical interfaces, reason and take autonomous, step-by-step action.</t>
         </is>
       </c>
+      <c r="U17" t="b">
+        <v>0</v>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>entity_linking</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>a third model (TML-Interaction / UI-TARS) beats both GPT and Gemini; GPT-4o and Gemini are not compared with each other</t>
+        </is>
+      </c>
       <c r="Y17" t="inlineStr">
         <is>
           <t>model:gpt_4o_2</t>
@@ -3242,6 +3440,24 @@
           <t>BEFORE: As evidenced by the tech giants’ recent announcements, the biggest AI players are unlikely to pull back on planned investments on DeepSeek’s account, Ashish Nadkarni, group vice president and general manager for worldwide infrastructure research at IDC, told Facilities Dive. || EVIDENCE: For companies like Meta and Microsoft, the drive to build as much AI capacity as quickly as possible is “ existential, ” with Apple the only major tech company to buck the trend so far, Nadkarni said. || AFTER: Those companies, and others like Elon Musk’s xAI, are using huge amounts of proprietary data to train differentiated foundational models useful in building emerging “ agentic AI ” tools and other future innovations, he added.</t>
         </is>
       </c>
+      <c r="U18" t="b">
+        <v>0</v>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>insufficient_context</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>Apple and Meta are penalized together for anti-competitive practices</t>
+        </is>
+      </c>
       <c r="Y18" t="inlineStr">
         <is>
           <t>org:apple</t>
@@ -3404,6 +3620,14 @@
 Performance: Claude Opus 5 leads many benchmarks at a cost per task lower than Claude Fable 5 but higher than most other models. || AFTER: The model’s widest performance margin came on a test of learning in unfamiliar environments.</t>
         </is>
       </c>
+      <c r="U19" t="b">
+        <v>1</v>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
       <c r="Y19" t="inlineStr">
         <is>
           <t>product:claude_opus_5</t>
@@ -3557,6 +3781,14 @@
 As people across the world spend increasing amounts of time interacting with chatbots like ChatGPT, chatbot makers are struggling to work out the kind of tone and “ personality ” the models should adopt. || EVIDENCE: Back in April, OpenAI admitted it’d struck the wrong balance between helpful and sniveling, saying a new update had rendered GPT-4o too sycophantic. || AFTER: Having it suck up to you isn’t just irritating—it can mislead users by reinforcing their incorrect beliefs and spreading misinformation.</t>
         </is>
       </c>
+      <c r="U20" t="b">
+        <v>1</v>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
       <c r="Y20" t="inlineStr">
         <is>
           <t>model:gpt_4o_2</t>
@@ -3717,6 +3949,14 @@
           <t>BEFORE: That’s where IBM’s Granite time series forecasting models fit in; they apply transformer technology to predict future values from time-based data. || EVIDENCE: “ Reasoning is not something a model is, it’s something a model does, ” David Cox, VP for AI models at IBM Research, told VentureBeat. || AFTER: While there has been no shortage of excitement and hype around reasoning models in 2025, reasoning for its own sake doesn’t necessarily provide value to enterprise users.</t>
         </is>
       </c>
+      <c r="U21" t="b">
+        <v>1</v>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
       <c r="Y21" t="inlineStr">
         <is>
           <t>person:david_cox</t>
@@ -3870,6 +4110,14 @@
 The Kimi research model even got a mention last week during Elon Musk's xAI release of Grok 4 — which scored 25.4 on its own on the "Humanity's Last Exam" benchmark, but attained a 44.4 score when allowed to use a variety of AI tools and web search.</t>
         </is>
       </c>
+      <c r="U22" t="b">
+        <v>1</v>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
       <c r="Y22" t="inlineStr">
         <is>
           <t>model:kimi</t>
@@ -4030,6 +4278,14 @@
           <t>BEFORE: In addition, it will be “ very interesting to see the use cases they uncover for the models, ” he says. || EVIDENCE: And as IBM’s Varshney sees it, geopolitical differences may also matter less than one might assume in this global AI race. || AFTER: “ Once a model is open-sourced, where it comes from stops mattering in many respects, ” he says.</t>
         </is>
       </c>
+      <c r="U23" t="b">
+        <v>1</v>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
       <c r="Y23" t="inlineStr">
         <is>
           <t>person:kush_varshney</t>
@@ -4177,6 +4433,14 @@
           <t>BEFORE: Nova Premier was announced as still in training, targeted for early 2025 release. || EVIDENCE: Yes — Amazon Nova Micro, Lite and Pro are all available on Amazon Bedrock, along with Amazon Nova Canvas and Reels. || AFTER: But Amazon Nova Premier will not be available until 2025.</t>
         </is>
       </c>
+      <c r="U24" t="b">
+        <v>1</v>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
       <c r="Y24" t="inlineStr">
         <is>
           <t>product:reels</t>
@@ -4325,6 +4589,14 @@
           <t>BEFORE: Before Monday’s GTC keynote with NVIDIA founder and CEO Jensen Huang, catch NVIDIA GTC Live — a preshow featuring analysts, founders and industry leaders shaping the next phase of AI — starting at 8 a.m. PT. || EVIDENCE: Hosts Sarah Guo, founder of AI-native investing firm Conviction; Gavin Baker, managing partner and chief investment officer of Atreides Management; and Alfred Lin, partner at Sequoia Capital, will talk with guests about the shift from general-purpose to accelerated computing and the five-layer foundation behind one of the largest infrastructure buildouts in history. || AFTER: Correspondent Tiffany Janzen, founder of TiffinTech, will chat with guests in the crowd — including a few notable tech leaders — to get live reactions.</t>
         </is>
       </c>
+      <c r="U25" t="b">
+        <v>1</v>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
       <c r="Y25" t="inlineStr">
         <is>
           <t>org:conviction</t>
@@ -4473,6 +4745,14 @@
           <t>BEFORE: Scale AI has made a business out of making Llama and Claude models from Anthropic consumable by and supportable for enterprises as well as providing tools to knock datasets into shape so they can feed into AI training runs. || EVIDENCE: Wang’s team brought over from Scale AI is one of the kernels of the Superintelligence Lab that Zuck &amp; Co have spent untold billions of dollars funding in the past year, bringing in fresh AI research talent and counterbalancing the loss of Yann LeCun, the long-time leader of the Facebook AI Research lab at New York University and one of the key researchers behind the development of the convolutional neural network more than four decades ago. || AFTER: (LeCun left FAIR a few weeks ago to start Advanced Machine Intelligence Labs, and has made no secret that he does not think the future of AI is GenAI LLMs.)</t>
         </is>
       </c>
+      <c r="U26" t="b">
+        <v>1</v>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
       <c r="Y26" t="inlineStr">
         <is>
           <t>person:yann_lecun</t>
@@ -4620,6 +4900,14 @@
           <t>BEFORE: Speeds and feeds are great, but hardware is only as useful as the software that can harness it, and, for AMD, that’s the ROCm software stack. || EVIDENCE: If you’re not familiar, ROCm is to AMD’s Instinct GPU accelerators what CUDA is to Nvidia GPUs. || AFTER: The respective software suites are essential to tapping into their hardware platform’s full potential, and ROCm is a particularly big one encompassing everything from drivers, development tools, libraries, and APIs necessary for running compute workloads on AMD kit.</t>
         </is>
       </c>
+      <c r="U27" t="b">
+        <v>1</v>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
       <c r="Y27" t="inlineStr">
         <is>
           <t>technology:rocm</t>
@@ -4772,6 +5060,14 @@
           <t>BEFORE: The liquid-cooled DGX SuperPod with DGX GB300 systems consists of eight GB300 NVL72 platforms, amounting to 288 Grace CPUs, 576 Blackwell Ultra GPUs and 300 TB of fast memory that can produce 11.4 exaflops of FP4 computation. || EVIDENCE: The DGX SuperPod with DGX B300 systems, on the other hand, is pitched by Nvidia as a “ scalable, air-cooled architecture ” that will be offered as a new design for the company’s modular MGX server racks and enterprise data centers. || AFTER: Nvidia provided a major road map update in March, saying that the company plans to release a rack-scale architecture for AI data centers that will connect 576 next-generation GPUs in the second half of 2027.</t>
         </is>
       </c>
+      <c r="U28" t="b">
+        <v>1</v>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
       <c r="Y28" t="inlineStr">
         <is>
           <t>product:dgx_superpod</t>
@@ -4932,6 +5228,24 @@
           <t>BEFORE: Its €600 million Series B in June 2024 pushed the valuation to nearly €6 billion, making it Europe’s highest-valued AI startup. || EVIDENCE: Major investors include General Catalyst, Andreessen Horowitz, Nvidia, Salesforce, IBM, and Microsoft, with Microsoft also partnering to distribute Mistral’s models through Azure. || AFTER: This robust financial backing and strategic partnerships have attracted prominent European clients like BNP Paribas, AXA, Stellantis, and CMA CGM, who value Mistral’s commitment to European data sovereignty and technical excellence.</t>
         </is>
       </c>
+      <c r="U29" t="b">
+        <v>0</v>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>entity_linking</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>Salesforce and Nvidia are co-investors in Mistral</t>
+        </is>
+      </c>
       <c r="Y29" t="inlineStr">
         <is>
           <t>org:salesforce</t>
@@ -5080,6 +5394,24 @@
           <t>BEFORE: Negative Sentiment: One market note also highlighted that Alibaba shares have lagged other major Chinese tech names this year, reflecting ongoing skepticism around Chinese internet stocks despite AI enthusiasm. || EVIDENCE: Here's why Alibaba, Tencent, Xiaomi stocks are falling amid the AI boom Analysts Set New Price || AFTER: TargetsA number of analysts have recently issued reports on BABA shares.</t>
         </is>
       </c>
+      <c r="U30" t="b">
+        <v>0</v>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>insufficient_context</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>Tencent and Xiaomi are only listed among China's big tech firms; no competition stated</t>
+        </is>
+      </c>
       <c r="Y30" t="inlineStr">
         <is>
           <t>org:tencent</t>
@@ -5230,6 +5562,21 @@
       <c r="T31" t="inlineStr">
         <is>
           <t>BEFORE: It was a message that he’s repeated this week at Nvidia’s GTC 2026 conference in San Jose, California. || EVIDENCE: For sure, there was been plenty of hardware talk during Huang’s keynote address during the show’s opening day, including platforms from Grace-Blackwell NVL72 to Vera-Rubin NVL72 to Nvidia’s plans for the Groq Language Processing Units (LPUs), not to mention storage systems and interconnects and the cloud business. || AFTER: But the overall focus of both the talk and the conference itself has been agentic AI, a market in which Nvidia is the dominant player, a position that Huang intends to keep and is willing spend a lot of money to ensure.</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>AMBIGUOUS</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>Reviewer_A</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>NVL72 is an NVIDIA platform ('NVIDIA Vera Rubin NVL72'), but nothing says NVIDIA manufactures it</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
@@ -10919,7 +11266,6 @@
           <t>jihyeon choung</t>
         </is>
       </c>
-      <c r="W64" t="inlineStr"/>
       <c r="Y64" t="inlineStr">
         <is>
           <t>model:o3_reasoning_model</t>
@@ -11082,7 +11428,6 @@
           <t>jihyeon choung</t>
         </is>
       </c>
-      <c r="W65" t="inlineStr"/>
       <c r="Y65" t="inlineStr">
         <is>
           <t>org:seed_club_ventures</t>
@@ -11245,7 +11590,6 @@
           <t>jihyeon choung</t>
         </is>
       </c>
-      <c r="W66" t="inlineStr"/>
       <c r="Y66" t="inlineStr">
         <is>
           <t>person:ashok_srivastava</t>
@@ -11411,7 +11755,6 @@
           <t>jihyeon choung</t>
         </is>
       </c>
-      <c r="W67" t="inlineStr"/>
       <c r="Y67" t="inlineStr">
         <is>
           <t>model:ling_2_5_1t</t>
@@ -11736,7 +12079,6 @@
           <t>jihyeon choung</t>
         </is>
       </c>
-      <c r="W69" t="inlineStr"/>
       <c r="Y69" t="inlineStr">
         <is>
           <t>org:open_source_alliance</t>
@@ -12069,7 +12411,6 @@
           <t>jihyeon choung</t>
         </is>
       </c>
-      <c r="W71" t="inlineStr"/>
       <c r="Y71" t="inlineStr">
         <is>
           <t>model:nim</t>
@@ -12241,7 +12582,6 @@
           <t>jihyeon choung</t>
         </is>
       </c>
-      <c r="W72" t="inlineStr"/>
       <c r="Y72" t="inlineStr">
         <is>
           <t>product:gemini_3</t>
@@ -12603,7 +12943,6 @@
           <t>jihyeon choung</t>
         </is>
       </c>
-      <c r="W74" t="inlineStr"/>
       <c r="Y74" t="inlineStr">
         <is>
           <t>org:openai</t>
@@ -13108,7 +13447,6 @@
           <t>jihyeon choung</t>
         </is>
       </c>
-      <c r="W77" t="inlineStr"/>
       <c r="Y77" t="inlineStr">
         <is>
           <t>model:weathernext</t>
@@ -13266,7 +13604,6 @@
           <t>jihyeon choung</t>
         </is>
       </c>
-      <c r="W78" t="inlineStr"/>
       <c r="Y78" t="inlineStr">
         <is>
           <t>product:ltx_2_3</t>
@@ -13781,7 +14118,6 @@
           <t>jihyeon choung</t>
         </is>
       </c>
-      <c r="W81" t="inlineStr"/>
       <c r="Y81" t="inlineStr">
         <is>
           <t>product:h20</t>
@@ -13951,7 +14287,6 @@
           <t>jihyeon choung</t>
         </is>
       </c>
-      <c r="W82" t="inlineStr"/>
       <c r="Y82" t="inlineStr">
         <is>
           <t>org:stability_ai</t>
@@ -14122,7 +14457,6 @@
           <t>jihyeon choung</t>
         </is>
       </c>
-      <c r="W83" t="inlineStr"/>
       <c r="Y83" t="inlineStr">
         <is>
           <t>product:spectrum_x_ethernet</t>
@@ -14615,7 +14949,6 @@
           <t>jihyeon choung</t>
         </is>
       </c>
-      <c r="W86" t="inlineStr"/>
       <c r="Y86" t="inlineStr">
         <is>
           <t>person:tomislav_pericin</t>
@@ -14943,7 +15276,6 @@
           <t>jihyeon choung</t>
         </is>
       </c>
-      <c r="W88" t="inlineStr"/>
       <c r="Y88" t="inlineStr">
         <is>
           <t>technology:cuopt</t>
@@ -15456,7 +15788,6 @@
           <t>jihyeon choung</t>
         </is>
       </c>
-      <c r="W91" t="inlineStr"/>
       <c r="Y91" t="inlineStr">
         <is>
           <t>org:windsurf</t>

</xml_diff>